<commit_message>
fix: make CSV reads round-trip exactly so exports are platform-stable
pandas' default fast float parser does not round-trip the last digit
and its rounding differs between CPU architectures. Re-reading the
pipeline export changed 283 of 330 lines, so notebook 09's report
drifted on Linux CI while staying stable on macOS.

io.read now defaults to float_precision='round_trip' for CSV/TSV. The
regenerated report_final.csv is byte-identical to the pipeline export and
report_final.parquet holds exactly the same values.
</commit_message>
<xml_diff>
--- a/exports/final_custom_styled.xlsx
+++ b/exports/final_custom_styled.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,16 +17,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="3">
@@ -42,7 +39,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -50,21 +47,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -435,44 +423,44 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>month</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>sales</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>profit</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>new_cases</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>hospitalized</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>rolling_profit</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>sales_pct_change</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="1" t="n">
+      <c r="A2" t="n">
         <v>0</v>
       </c>
       <c r="B2" t="inlineStr">
@@ -496,7 +484,7 @@
       <c r="H2" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" s="1" t="n">
+      <c r="A3" t="n">
         <v>1</v>
       </c>
       <c r="B3" t="inlineStr">
@@ -522,7 +510,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="1" t="n">
+      <c r="A4" t="n">
         <v>2</v>
       </c>
       <c r="B4" t="inlineStr">
@@ -550,7 +538,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="1" t="n">
+      <c r="A5" t="n">
         <v>3</v>
       </c>
       <c r="B5" t="inlineStr">
@@ -578,7 +566,7 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="1" t="n">
+      <c r="A6" t="n">
         <v>4</v>
       </c>
       <c r="B6" t="inlineStr">
@@ -602,11 +590,11 @@
         <v>1412.426666666667</v>
       </c>
       <c r="H6" t="n">
-        <v>0.2751046753549648</v>
+        <v>0.2751046753549649</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="1" t="n">
+      <c r="A7" t="n">
         <v>5</v>
       </c>
       <c r="B7" t="inlineStr">
@@ -630,11 +618,11 @@
         <v>1345.693333333333</v>
       </c>
       <c r="H7" t="n">
-        <v>-0.038760539165786</v>
+        <v>-0.03876053916578603</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="1" t="n">
+      <c r="A8" t="n">
         <v>6</v>
       </c>
       <c r="B8" t="inlineStr">
@@ -658,11 +646,11 @@
         <v>1496.94</v>
       </c>
       <c r="H8" t="n">
-        <v>-0.0044555851817584</v>
+        <v>-0.004455585181758481</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="1" t="n">
+      <c r="A9" t="n">
         <v>7</v>
       </c>
       <c r="B9" t="inlineStr">
@@ -686,11 +674,11 @@
         <v>1414.093333333333</v>
       </c>
       <c r="H9" t="n">
-        <v>0.0683249719034342</v>
+        <v>0.06832497190343423</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="1" t="n">
+      <c r="A10" t="n">
         <v>8</v>
       </c>
       <c r="B10" t="inlineStr">
@@ -714,11 +702,11 @@
         <v>1598.7</v>
       </c>
       <c r="H10" t="n">
-        <v>-0.0697187107737816</v>
+        <v>-0.06971871077378167</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="1" t="n">
+      <c r="A11" t="n">
         <v>9</v>
       </c>
       <c r="B11" t="inlineStr">
@@ -742,11 +730,11 @@
         <v>1574.87</v>
       </c>
       <c r="H11" t="n">
-        <v>0.0135243730595793</v>
+        <v>0.01352437305957932</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="1" t="n">
+      <c r="A12" t="n">
         <v>10</v>
       </c>
       <c r="B12" t="inlineStr">
@@ -774,7 +762,7 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="1" t="n">
+      <c r="A13" t="n">
         <v>11</v>
       </c>
       <c r="B13" t="inlineStr">
@@ -798,11 +786,11 @@
         <v>1555.88</v>
       </c>
       <c r="H13" t="n">
-        <v>-0.0156722842854944</v>
+        <v>-0.0156722842854945</v>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="1" t="n">
+      <c r="A14" t="n">
         <v>12</v>
       </c>
       <c r="B14" t="inlineStr">
@@ -826,11 +814,11 @@
         <v>1542.976666666667</v>
       </c>
       <c r="H14" t="n">
-        <v>-0.0746022858078195</v>
+        <v>-0.07460228580781958</v>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="1" t="n">
+      <c r="A15" t="n">
         <v>13</v>
       </c>
       <c r="B15" t="inlineStr">
@@ -854,11 +842,11 @@
         <v>1449.866666666667</v>
       </c>
       <c r="H15" t="n">
-        <v>-0.0807790218039319</v>
+        <v>-0.08077902180393193</v>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="1" t="n">
+      <c r="A16" t="n">
         <v>14</v>
       </c>
       <c r="B16" t="inlineStr">
@@ -882,11 +870,11 @@
         <v>1414.336666666667</v>
       </c>
       <c r="H16" t="n">
-        <v>-0.0109719501124604</v>
+        <v>-0.01097195011246044</v>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="1" t="n">
+      <c r="A17" t="n">
         <v>15</v>
       </c>
       <c r="B17" t="inlineStr">
@@ -910,11 +898,11 @@
         <v>1299.576666666667</v>
       </c>
       <c r="H17" t="n">
-        <v>0.0444786048913903</v>
+        <v>0.04447860489139033</v>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="1" t="n">
+      <c r="A18" t="n">
         <v>16</v>
       </c>
       <c r="B18" t="inlineStr">
@@ -932,17 +920,17 @@
         <v>15482</v>
       </c>
       <c r="F18" t="n">
-        <v>2562.290322580646</v>
+        <v>2562.290322580645</v>
       </c>
       <c r="G18" t="n">
         <v>1259.753333333333</v>
       </c>
       <c r="H18" t="n">
-        <v>0.0206304137708068</v>
+        <v>0.02063041377080688</v>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="1" t="n">
+      <c r="A19" t="n">
         <v>17</v>
       </c>
       <c r="B19" t="inlineStr">
@@ -966,11 +954,11 @@
         <v>1359.66</v>
       </c>
       <c r="H19" t="n">
-        <v>0.0438153466796042</v>
+        <v>0.04381534667960429</v>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="1" t="n">
+      <c r="A20" t="n">
         <v>18</v>
       </c>
       <c r="B20" t="inlineStr">
@@ -994,11 +982,11 @@
         <v>1460.583333333333</v>
       </c>
       <c r="H20" t="n">
-        <v>-0.0472335039348412</v>
+        <v>-0.04723350393484127</v>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="1" t="n">
+      <c r="A21" t="n">
         <v>19</v>
       </c>
       <c r="B21" t="inlineStr">
@@ -1022,11 +1010,11 @@
         <v>1579.046666666666</v>
       </c>
       <c r="H21" t="n">
-        <v>-0.0250709140034445</v>
+        <v>-0.02507091400344452</v>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="1" t="n">
+      <c r="A22" t="n">
         <v>20</v>
       </c>
       <c r="B22" t="inlineStr">
@@ -1050,11 +1038,11 @@
         <v>1336.15</v>
       </c>
       <c r="H22" t="n">
-        <v>0.0316114874289381</v>
+        <v>0.03161148742893816</v>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="1" t="n">
+      <c r="A23" t="n">
         <v>21</v>
       </c>
       <c r="B23" t="inlineStr">
@@ -1078,11 +1066,11 @@
         <v>1450.453333333334</v>
       </c>
       <c r="H23" t="n">
-        <v>0.0700233431928485</v>
+        <v>0.07002334319284853</v>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="1" t="n">
+      <c r="A24" t="n">
         <v>22</v>
       </c>
       <c r="B24" t="inlineStr">
@@ -1106,11 +1094,11 @@
         <v>1517.216666666666</v>
       </c>
       <c r="H24" t="n">
-        <v>0.0704257490848063</v>
+        <v>0.07042574908480637</v>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="1" t="n">
+      <c r="A25" t="n">
         <v>23</v>
       </c>
       <c r="B25" t="inlineStr">
@@ -1134,11 +1122,11 @@
         <v>1615.16</v>
       </c>
       <c r="H25" t="n">
-        <v>-0.13932437016781</v>
+        <v>-0.1393243701678101</v>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="1" t="n">
+      <c r="A26" t="n">
         <v>24</v>
       </c>
       <c r="B26" t="inlineStr">
@@ -1166,7 +1154,7 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="1" t="n">
+      <c r="A27" t="n">
         <v>25</v>
       </c>
       <c r="B27" t="inlineStr">
@@ -1194,7 +1182,7 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="1" t="n">
+      <c r="A28" t="n">
         <v>26</v>
       </c>
       <c r="B28" t="inlineStr">
@@ -1222,7 +1210,7 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="1" t="n">
+      <c r="A29" t="n">
         <v>27</v>
       </c>
       <c r="B29" t="inlineStr">
@@ -1250,7 +1238,7 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="1" t="n">
+      <c r="A30" t="n">
         <v>28</v>
       </c>
       <c r="B30" t="inlineStr">
@@ -1278,7 +1266,7 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="1" t="n">
+      <c r="A31" t="n">
         <v>29</v>
       </c>
       <c r="B31" t="inlineStr">
@@ -1306,7 +1294,7 @@
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="1" t="n">
+      <c r="A32" t="n">
         <v>30</v>
       </c>
       <c r="B32" t="inlineStr">
@@ -1330,11 +1318,11 @@
         <v>1317.633333333333</v>
       </c>
       <c r="H32" t="n">
-        <v>-0.1366383140789639</v>
+        <v>-0.136638314078964</v>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="1" t="n">
+      <c r="A33" t="n">
         <v>31</v>
       </c>
       <c r="B33" t="inlineStr">
@@ -1358,11 +1346,11 @@
         <v>1201.97</v>
       </c>
       <c r="H33" t="n">
-        <v>-0.1098144628334296</v>
+        <v>-0.1098144628334297</v>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="1" t="n">
+      <c r="A34" t="n">
         <v>32</v>
       </c>
       <c r="B34" t="inlineStr">
@@ -1386,11 +1374,11 @@
         <v>1299.053333333333</v>
       </c>
       <c r="H34" t="n">
-        <v>0.0973011580418898</v>
+        <v>0.09730115804188988</v>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="1" t="n">
+      <c r="A35" t="n">
         <v>33</v>
       </c>
       <c r="B35" t="inlineStr">
@@ -1418,7 +1406,7 @@
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="1" t="n">
+      <c r="A36" t="n">
         <v>34</v>
       </c>
       <c r="B36" t="inlineStr">
@@ -1446,7 +1434,7 @@
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="1" t="n">
+      <c r="A37" t="n">
         <v>35</v>
       </c>
       <c r="B37" t="inlineStr">
@@ -1474,7 +1462,7 @@
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="1" t="n">
+      <c r="A38" t="n">
         <v>36</v>
       </c>
       <c r="B38" t="inlineStr">
@@ -1498,11 +1486,11 @@
         <v>1424.31</v>
       </c>
       <c r="H38" t="n">
-        <v>0.0289242088693062</v>
+        <v>0.02892420886930624</v>
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="1" t="n">
+      <c r="A39" t="n">
         <v>37</v>
       </c>
       <c r="B39" t="inlineStr">
@@ -1530,7 +1518,7 @@
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="1" t="n">
+      <c r="A40" t="n">
         <v>38</v>
       </c>
       <c r="B40" t="inlineStr">
@@ -1558,7 +1546,7 @@
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="1" t="n">
+      <c r="A41" t="n">
         <v>39</v>
       </c>
       <c r="B41" t="inlineStr">
@@ -1582,11 +1570,11 @@
         <v>1276.506666666667</v>
       </c>
       <c r="H41" t="n">
-        <v>-0.08542283072476591</v>
+        <v>-0.08542283072476597</v>
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="1" t="n">
+      <c r="A42" t="n">
         <v>40</v>
       </c>
       <c r="B42" t="inlineStr">
@@ -1614,7 +1602,7 @@
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="1" t="n">
+      <c r="A43" t="n">
         <v>41</v>
       </c>
       <c r="B43" t="inlineStr">
@@ -1642,7 +1630,7 @@
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="1" t="n">
+      <c r="A44" t="n">
         <v>42</v>
       </c>
       <c r="B44" t="inlineStr">
@@ -1670,7 +1658,7 @@
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="1" t="n">
+      <c r="A45" t="n">
         <v>43</v>
       </c>
       <c r="B45" t="inlineStr">
@@ -1698,7 +1686,7 @@
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="1" t="n">
+      <c r="A46" t="n">
         <v>44</v>
       </c>
       <c r="B46" t="inlineStr">
@@ -1726,7 +1714,7 @@
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="1" t="n">
+      <c r="A47" t="n">
         <v>45</v>
       </c>
       <c r="B47" t="inlineStr">
@@ -1750,11 +1738,11 @@
         <v>1741.716666666667</v>
       </c>
       <c r="H47" t="n">
-        <v>0.2468512759010985</v>
+        <v>0.2468512759010986</v>
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="1" t="n">
+      <c r="A48" t="n">
         <v>46</v>
       </c>
       <c r="B48" t="inlineStr">
@@ -1782,7 +1770,7 @@
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="1" t="n">
+      <c r="A49" t="n">
         <v>47</v>
       </c>
       <c r="B49" t="inlineStr">
@@ -1794,7 +1782,7 @@
         <v>29356.68</v>
       </c>
       <c r="D49" t="n">
-        <v>929.41</v>
+        <v>929.4100000000001</v>
       </c>
       <c r="E49" t="n">
         <v>15359</v>
@@ -1806,11 +1794,11 @@
         <v>1571.206666666667</v>
       </c>
       <c r="H49" t="n">
-        <v>-0.0665982433783298</v>
+        <v>-0.06659824337832987</v>
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="1" t="n">
+      <c r="A50" t="n">
         <v>48</v>
       </c>
       <c r="B50" t="inlineStr">
@@ -1838,7 +1826,7 @@
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="1" t="n">
+      <c r="A51" t="n">
         <v>49</v>
       </c>
       <c r="B51" t="inlineStr">
@@ -1862,11 +1850,11 @@
         <v>1112.06</v>
       </c>
       <c r="H51" t="n">
-        <v>-0.1985100808412818</v>
+        <v>-0.1985100808412819</v>
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="1" t="n">
+      <c r="A52" t="n">
         <v>50</v>
       </c>
       <c r="B52" t="inlineStr">
@@ -1887,14 +1875,14 @@
         <v>2367.548387096774</v>
       </c>
       <c r="G52" t="n">
-        <v>1236.353333333334</v>
+        <v>1236.353333333333</v>
       </c>
       <c r="H52" t="n">
-        <v>0.07635726305661419</v>
+        <v>0.07635726305661428</v>
       </c>
     </row>
     <row r="53">
-      <c r="A53" s="1" t="n">
+      <c r="A53" t="n">
         <v>51</v>
       </c>
       <c r="B53" t="inlineStr">
@@ -1922,7 +1910,7 @@
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="1" t="n">
+      <c r="A54" t="n">
         <v>52</v>
       </c>
       <c r="B54" t="inlineStr">
@@ -1940,17 +1928,17 @@
         <v>15470</v>
       </c>
       <c r="F54" t="n">
-        <v>2805.709677419354</v>
+        <v>2805.709677419355</v>
       </c>
       <c r="G54" t="n">
         <v>1529.213333333333</v>
       </c>
       <c r="H54" t="n">
-        <v>0.0159162543768915</v>
+        <v>0.01591625437689159</v>
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="1" t="n">
+      <c r="A55" t="n">
         <v>53</v>
       </c>
       <c r="B55" t="inlineStr">
@@ -1978,7 +1966,7 @@
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="1" t="n">
+      <c r="A56" t="n">
         <v>54</v>
       </c>
       <c r="B56" t="inlineStr">
@@ -2002,11 +1990,11 @@
         <v>1565.996666666667</v>
       </c>
       <c r="H56" t="n">
-        <v>0.0064166556620588</v>
+        <v>0.006416655662058846</v>
       </c>
     </row>
     <row r="57">
-      <c r="A57" s="1" t="n">
+      <c r="A57" t="n">
         <v>55</v>
       </c>
       <c r="B57" t="inlineStr">
@@ -2030,11 +2018,11 @@
         <v>1640.736666666667</v>
       </c>
       <c r="H57" t="n">
-        <v>0.07105066534682811</v>
+        <v>0.07105066534682813</v>
       </c>
     </row>
     <row r="58">
-      <c r="A58" s="1" t="n">
+      <c r="A58" t="n">
         <v>56</v>
       </c>
       <c r="B58" t="inlineStr">
@@ -2058,11 +2046,11 @@
         <v>1760.283333333334</v>
       </c>
       <c r="H58" t="n">
-        <v>-0.0745321251280234</v>
+        <v>-0.07453212512802343</v>
       </c>
     </row>
     <row r="59">
-      <c r="A59" s="1" t="n">
+      <c r="A59" t="n">
         <v>57</v>
       </c>
       <c r="B59" t="inlineStr">
@@ -2090,7 +2078,7 @@
       </c>
     </row>
     <row r="60">
-      <c r="A60" s="1" t="n">
+      <c r="A60" t="n">
         <v>58</v>
       </c>
       <c r="B60" t="inlineStr">
@@ -2114,11 +2102,11 @@
         <v>1751.076666666667</v>
       </c>
       <c r="H60" t="n">
-        <v>-0.0027450474781328</v>
+        <v>-0.002745047478132867</v>
       </c>
     </row>
     <row r="61">
-      <c r="A61" s="1" t="n">
+      <c r="A61" t="n">
         <v>59</v>
       </c>
       <c r="B61" t="inlineStr">
@@ -2142,11 +2130,11 @@
         <v>1779.423333333333</v>
       </c>
       <c r="H61" t="n">
-        <v>-0.0678846038497912</v>
+        <v>-0.06788460384979123</v>
       </c>
     </row>
     <row r="62">
-      <c r="A62" s="1" t="n">
+      <c r="A62" t="n">
         <v>60</v>
       </c>
       <c r="B62" t="inlineStr">
@@ -2174,7 +2162,7 @@
       </c>
     </row>
     <row r="63">
-      <c r="A63" s="1" t="n">
+      <c r="A63" t="n">
         <v>61</v>
       </c>
       <c r="B63" t="inlineStr">
@@ -2198,11 +2186,11 @@
         <v>1744.056666666667</v>
       </c>
       <c r="H63" t="n">
-        <v>-0.0838145614746971</v>
+        <v>-0.08381456147469712</v>
       </c>
     </row>
     <row r="64">
-      <c r="A64" s="1" t="n">
+      <c r="A64" t="n">
         <v>62</v>
       </c>
       <c r="B64" t="inlineStr">
@@ -2226,11 +2214,11 @@
         <v>1919.976666666667</v>
       </c>
       <c r="H64" t="n">
-        <v>0.0275841080561576</v>
+        <v>0.02758410805615763</v>
       </c>
     </row>
     <row r="65">
-      <c r="A65" s="1" t="n">
+      <c r="A65" t="n">
         <v>63</v>
       </c>
       <c r="B65" t="inlineStr">
@@ -2254,11 +2242,11 @@
         <v>1704.23</v>
       </c>
       <c r="H65" t="n">
-        <v>-0.1277950333983227</v>
+        <v>-0.1277950333983228</v>
       </c>
     </row>
     <row r="66">
-      <c r="A66" s="1" t="n">
+      <c r="A66" t="n">
         <v>64</v>
       </c>
       <c r="B66" t="inlineStr">
@@ -2282,11 +2270,11 @@
         <v>1538.950000000001</v>
       </c>
       <c r="H66" t="n">
-        <v>0.2306192733006224</v>
+        <v>0.2306192733006225</v>
       </c>
     </row>
     <row r="67">
-      <c r="A67" s="1" t="n">
+      <c r="A67" t="n">
         <v>65</v>
       </c>
       <c r="B67" t="inlineStr">
@@ -2314,7 +2302,7 @@
       </c>
     </row>
     <row r="68">
-      <c r="A68" s="1" t="n">
+      <c r="A68" t="n">
         <v>66</v>
       </c>
       <c r="B68" t="inlineStr">
@@ -2342,7 +2330,7 @@
       </c>
     </row>
     <row r="69">
-      <c r="A69" s="1" t="n">
+      <c r="A69" t="n">
         <v>67</v>
       </c>
       <c r="B69" t="inlineStr">
@@ -2366,11 +2354,11 @@
         <v>1685.393333333334</v>
       </c>
       <c r="H69" t="n">
-        <v>0.1438357930334641</v>
+        <v>0.1438357930334642</v>
       </c>
     </row>
     <row r="70">
-      <c r="A70" s="1" t="n">
+      <c r="A70" t="n">
         <v>68</v>
       </c>
       <c r="B70" t="inlineStr">
@@ -2398,7 +2386,7 @@
       </c>
     </row>
     <row r="71">
-      <c r="A71" s="1" t="n">
+      <c r="A71" t="n">
         <v>69</v>
       </c>
       <c r="B71" t="inlineStr">
@@ -2422,11 +2410,11 @@
         <v>1906.88</v>
       </c>
       <c r="H71" t="n">
-        <v>0.0381327434393732</v>
+        <v>0.03813274343937323</v>
       </c>
     </row>
     <row r="72">
-      <c r="A72" s="1" t="n">
+      <c r="A72" t="n">
         <v>70</v>
       </c>
       <c r="B72" t="inlineStr">
@@ -2454,7 +2442,7 @@
       </c>
     </row>
     <row r="73">
-      <c r="A73" s="1" t="n">
+      <c r="A73" t="n">
         <v>71</v>
       </c>
       <c r="B73" t="inlineStr">
@@ -2482,7 +2470,7 @@
       </c>
     </row>
     <row r="74">
-      <c r="A74" s="1" t="n">
+      <c r="A74" t="n">
         <v>72</v>
       </c>
       <c r="B74" t="inlineStr">
@@ -2506,11 +2494,11 @@
         <v>1606.553333333334</v>
       </c>
       <c r="H74" t="n">
-        <v>-0.0216893216267085</v>
+        <v>-0.02168932162670856</v>
       </c>
     </row>
     <row r="75">
-      <c r="A75" s="1" t="n">
+      <c r="A75" t="n">
         <v>73</v>
       </c>
       <c r="B75" t="inlineStr">
@@ -2534,11 +2522,11 @@
         <v>1752.526666666667</v>
       </c>
       <c r="H75" t="n">
-        <v>-0.0583223587132061</v>
+        <v>-0.05832235871320612</v>
       </c>
     </row>
     <row r="76">
-      <c r="A76" s="1" t="n">
+      <c r="A76" t="n">
         <v>74</v>
       </c>
       <c r="B76" t="inlineStr">
@@ -2562,11 +2550,11 @@
         <v>1879.226666666667</v>
       </c>
       <c r="H76" t="n">
-        <v>0.0198043436967905</v>
+        <v>0.01980434369679052</v>
       </c>
     </row>
     <row r="77">
-      <c r="A77" s="1" t="n">
+      <c r="A77" t="n">
         <v>75</v>
       </c>
       <c r="B77" t="inlineStr">
@@ -2590,11 +2578,11 @@
         <v>1719.000000000001</v>
       </c>
       <c r="H77" t="n">
-        <v>-0.1065531367906152</v>
+        <v>-0.1065531367906153</v>
       </c>
     </row>
     <row r="78">
-      <c r="A78" s="1" t="n">
+      <c r="A78" t="n">
         <v>76</v>
       </c>
       <c r="B78" t="inlineStr">
@@ -2618,11 +2606,11 @@
         <v>1736.453333333334</v>
       </c>
       <c r="H78" t="n">
-        <v>0.1035422322927683</v>
+        <v>0.1035422322927684</v>
       </c>
     </row>
     <row r="79">
-      <c r="A79" s="1" t="n">
+      <c r="A79" t="n">
         <v>77</v>
       </c>
       <c r="B79" t="inlineStr">
@@ -2650,7 +2638,7 @@
       </c>
     </row>
     <row r="80">
-      <c r="A80" s="1" t="n">
+      <c r="A80" t="n">
         <v>78</v>
       </c>
       <c r="B80" t="inlineStr">
@@ -2678,7 +2666,7 @@
       </c>
     </row>
     <row r="81">
-      <c r="A81" s="1" t="n">
+      <c r="A81" t="n">
         <v>79</v>
       </c>
       <c r="B81" t="inlineStr">
@@ -2696,7 +2684,7 @@
         <v>15569</v>
       </c>
       <c r="F81" t="n">
-        <v>2738.290322580646</v>
+        <v>2738.290322580645</v>
       </c>
       <c r="G81" t="n">
         <v>1812.376666666667</v>
@@ -2706,7 +2694,7 @@
       </c>
     </row>
     <row r="82">
-      <c r="A82" s="1" t="n">
+      <c r="A82" t="n">
         <v>80</v>
       </c>
       <c r="B82" t="inlineStr">
@@ -2730,11 +2718,11 @@
         <v>1618.086666666667</v>
       </c>
       <c r="H82" t="n">
-        <v>-0.0367845006717949</v>
+        <v>-0.03678450067179495</v>
       </c>
     </row>
     <row r="83">
-      <c r="A83" s="1" t="n">
+      <c r="A83" t="n">
         <v>81</v>
       </c>
       <c r="B83" t="inlineStr">
@@ -2758,11 +2746,11 @@
         <v>1707.496666666667</v>
       </c>
       <c r="H83" t="n">
-        <v>-0.2835664716324659</v>
+        <v>-0.283566471632466</v>
       </c>
     </row>
     <row r="84">
-      <c r="A84" s="1" t="n">
+      <c r="A84" t="n">
         <v>82</v>
       </c>
       <c r="B84" t="inlineStr">
@@ -2786,11 +2774,11 @@
         <v>1598.353333333334</v>
       </c>
       <c r="H84" t="n">
-        <v>0.1251635238687287</v>
+        <v>0.1251635238687288</v>
       </c>
     </row>
     <row r="85">
-      <c r="A85" s="1" t="n">
+      <c r="A85" t="n">
         <v>83</v>
       </c>
       <c r="B85" t="inlineStr">
@@ -2808,17 +2796,17 @@
         <v>15669</v>
       </c>
       <c r="F85" t="n">
-        <v>2621.709677419354</v>
+        <v>2621.709677419355</v>
       </c>
       <c r="G85" t="n">
         <v>1326.700000000001</v>
       </c>
       <c r="H85" t="n">
-        <v>-0.06425699972281999</v>
+        <v>-0.06425699972282006</v>
       </c>
     </row>
     <row r="86">
-      <c r="A86" s="1" t="n">
+      <c r="A86" t="n">
         <v>84</v>
       </c>
       <c r="B86" t="inlineStr">
@@ -2846,7 +2834,7 @@
       </c>
     </row>
     <row r="87">
-      <c r="A87" s="1" t="n">
+      <c r="A87" t="n">
         <v>85</v>
       </c>
       <c r="B87" t="inlineStr">
@@ -2874,7 +2862,7 @@
       </c>
     </row>
     <row r="88">
-      <c r="A88" s="1" t="n">
+      <c r="A88" t="n">
         <v>86</v>
       </c>
       <c r="B88" t="inlineStr">
@@ -2898,11 +2886,11 @@
         <v>1476.74</v>
       </c>
       <c r="H88" t="n">
-        <v>0.1397469340821728</v>
+        <v>0.1397469340821729</v>
       </c>
     </row>
     <row r="89">
-      <c r="A89" s="1" t="n">
+      <c r="A89" t="n">
         <v>87</v>
       </c>
       <c r="B89" t="inlineStr">
@@ -2926,11 +2914,11 @@
         <v>1799.26</v>
       </c>
       <c r="H89" t="n">
-        <v>-0.0725562655962457</v>
+        <v>-0.07255626559624573</v>
       </c>
     </row>
     <row r="90">
-      <c r="A90" s="1" t="n">
+      <c r="A90" t="n">
         <v>88</v>
       </c>
       <c r="B90" t="inlineStr">
@@ -2954,11 +2942,11 @@
         <v>1894.156666666667</v>
       </c>
       <c r="H90" t="n">
-        <v>0.008495682966540999</v>
+        <v>0.008495682966541018</v>
       </c>
     </row>
     <row r="91">
-      <c r="A91" s="1" t="n">
+      <c r="A91" t="n">
         <v>89</v>
       </c>
       <c r="B91" t="inlineStr">
@@ -2986,7 +2974,7 @@
       </c>
     </row>
     <row r="92">
-      <c r="A92" s="1" t="n">
+      <c r="A92" t="n">
         <v>90</v>
       </c>
       <c r="B92" t="inlineStr">
@@ -3010,11 +2998,11 @@
         <v>1752.113333333334</v>
       </c>
       <c r="H92" t="n">
-        <v>0.1939116581740478</v>
+        <v>0.1939116581740479</v>
       </c>
     </row>
     <row r="93">
-      <c r="A93" s="1" t="n">
+      <c r="A93" t="n">
         <v>91</v>
       </c>
       <c r="B93" t="inlineStr">
@@ -3038,11 +3026,11 @@
         <v>1834.373333333334</v>
       </c>
       <c r="H93" t="n">
-        <v>0.0378290054950642</v>
+        <v>0.03782900549506429</v>
       </c>
     </row>
     <row r="94">
-      <c r="A94" s="1" t="n">
+      <c r="A94" t="n">
         <v>92</v>
       </c>
       <c r="B94" t="inlineStr">
@@ -3053,7 +3041,7 @@
       <c r="C94" t="n">
         <v>32937.1</v>
       </c>
-      <c r="D94" s="2" t="n">
+      <c r="D94" s="1" t="n">
         <v>2638.83</v>
       </c>
       <c r="E94" t="n">
@@ -3062,15 +3050,15 @@
       <c r="F94" t="n">
         <v>2345.066666666667</v>
       </c>
-      <c r="G94" s="2" t="n">
+      <c r="G94" s="1" t="n">
         <v>2277.846666666667</v>
       </c>
       <c r="H94" t="n">
-        <v>-0.0246948053467065</v>
+        <v>-0.02469480534670654</v>
       </c>
     </row>
     <row r="95">
-      <c r="A95" s="1" t="n">
+      <c r="A95" t="n">
         <v>93</v>
       </c>
       <c r="B95" t="inlineStr">
@@ -3094,11 +3082,11 @@
         <v>1926.556666666667</v>
       </c>
       <c r="H95" t="n">
-        <v>-0.0442771221510089</v>
+        <v>-0.04427712215100899</v>
       </c>
     </row>
     <row r="96">
-      <c r="A96" s="1" t="n">
+      <c r="A96" t="n">
         <v>94</v>
       </c>
       <c r="B96" t="inlineStr">
@@ -3126,7 +3114,7 @@
       </c>
     </row>
     <row r="97">
-      <c r="A97" s="1" t="n">
+      <c r="A97" t="n">
         <v>95</v>
       </c>
       <c r="B97" t="inlineStr">
@@ -3150,11 +3138,11 @@
         <v>1243.580000000001</v>
       </c>
       <c r="H97" t="n">
-        <v>0.0292113963265647</v>
+        <v>0.02921139632656478</v>
       </c>
     </row>
     <row r="98">
-      <c r="A98" s="1" t="n">
+      <c r="A98" t="n">
         <v>96</v>
       </c>
       <c r="B98" t="inlineStr">
@@ -3172,7 +3160,7 @@
         <v>15535</v>
       </c>
       <c r="F98" t="n">
-        <v>2182.709677419354</v>
+        <v>2182.709677419355</v>
       </c>
       <c r="G98" t="n">
         <v>1364.063333333334</v>
@@ -3182,7 +3170,7 @@
       </c>
     </row>
     <row r="99">
-      <c r="A99" s="1" t="n">
+      <c r="A99" t="n">
         <v>97</v>
       </c>
       <c r="B99" t="inlineStr">
@@ -3203,14 +3191,14 @@
         <v>2506</v>
       </c>
       <c r="G99" t="n">
-        <v>1388.593333333334</v>
+        <v>1388.593333333333</v>
       </c>
       <c r="H99" t="n">
         <v>-0.083722378820138</v>
       </c>
     </row>
     <row r="100">
-      <c r="A100" s="1" t="n">
+      <c r="A100" t="n">
         <v>98</v>
       </c>
       <c r="B100" t="inlineStr">
@@ -3228,17 +3216,17 @@
         <v>15688</v>
       </c>
       <c r="F100" t="n">
-        <v>2255.290322580646</v>
+        <v>2255.290322580645</v>
       </c>
       <c r="G100" t="n">
         <v>1582.156666666667</v>
       </c>
       <c r="H100" t="n">
-        <v>-0.0095265884578398</v>
+        <v>-0.009526588457839824</v>
       </c>
     </row>
     <row r="101">
-      <c r="A101" s="1" t="n">
+      <c r="A101" t="n">
         <v>99</v>
       </c>
       <c r="B101" t="inlineStr">
@@ -3266,7 +3254,7 @@
       </c>
     </row>
     <row r="102">
-      <c r="A102" s="1" t="n">
+      <c r="A102" t="n">
         <v>100</v>
       </c>
       <c r="B102" t="inlineStr">
@@ -3290,11 +3278,11 @@
         <v>1522.703333333334</v>
       </c>
       <c r="H102" t="n">
-        <v>-0.0612097997701899</v>
+        <v>-0.06120979977018992</v>
       </c>
     </row>
     <row r="103">
-      <c r="A103" s="1" t="n">
+      <c r="A103" t="n">
         <v>101</v>
       </c>
       <c r="B103" t="inlineStr">
@@ -3318,11 +3306,11 @@
         <v>1259.113333333334</v>
       </c>
       <c r="H103" t="n">
-        <v>-0.0372303641158682</v>
+        <v>-0.03723036411586822</v>
       </c>
     </row>
     <row r="104">
-      <c r="A104" s="1" t="n">
+      <c r="A104" t="n">
         <v>102</v>
       </c>
       <c r="B104" t="inlineStr">
@@ -3340,17 +3328,17 @@
         <v>15341</v>
       </c>
       <c r="F104" t="n">
-        <v>2565.709677419354</v>
+        <v>2565.709677419355</v>
       </c>
       <c r="G104" t="n">
         <v>1062.303333333334</v>
       </c>
       <c r="H104" t="n">
-        <v>0.0700669368035262</v>
+        <v>0.07006693680352627</v>
       </c>
     </row>
     <row r="105">
-      <c r="A105" s="1" t="n">
+      <c r="A105" t="n">
         <v>103</v>
       </c>
       <c r="B105" t="inlineStr">
@@ -3374,11 +3362,11 @@
         <v>1211.276666666667</v>
       </c>
       <c r="H105" t="n">
-        <v>0.0251082155160389</v>
+        <v>0.02510821551603892</v>
       </c>
     </row>
     <row r="106">
-      <c r="A106" s="1" t="n">
+      <c r="A106" t="n">
         <v>104</v>
       </c>
       <c r="B106" t="inlineStr">
@@ -3402,11 +3390,11 @@
         <v>1425.426666666667</v>
       </c>
       <c r="H106" t="n">
-        <v>-0.0550641622668018</v>
+        <v>-0.05506416226680189</v>
       </c>
     </row>
     <row r="107">
-      <c r="A107" s="1" t="n">
+      <c r="A107" t="n">
         <v>105</v>
       </c>
       <c r="B107" t="inlineStr">
@@ -3434,7 +3422,7 @@
       </c>
     </row>
     <row r="108">
-      <c r="A108" s="1" t="n">
+      <c r="A108" t="n">
         <v>106</v>
       </c>
       <c r="B108" t="inlineStr">
@@ -3462,7 +3450,7 @@
       </c>
     </row>
     <row r="109">
-      <c r="A109" s="1" t="n">
+      <c r="A109" t="n">
         <v>107</v>
       </c>
       <c r="B109" t="inlineStr">
@@ -3486,11 +3474,11 @@
         <v>1638.306666666667</v>
       </c>
       <c r="H109" t="n">
-        <v>0.0095435266470336</v>
+        <v>0.009543526647033618</v>
       </c>
     </row>
     <row r="110">
-      <c r="A110" s="1" t="n">
+      <c r="A110" t="n">
         <v>108</v>
       </c>
       <c r="B110" t="inlineStr">
@@ -3514,11 +3502,11 @@
         <v>1736.116666666667</v>
       </c>
       <c r="H110" t="n">
-        <v>-0.038639367884955</v>
+        <v>-0.03863936788495503</v>
       </c>
     </row>
     <row r="111">
-      <c r="A111" s="1" t="n">
+      <c r="A111" t="n">
         <v>109</v>
       </c>
       <c r="B111" t="inlineStr">
@@ -3546,7 +3534,7 @@
       </c>
     </row>
     <row r="112">
-      <c r="A112" s="1" t="n">
+      <c r="A112" t="n">
         <v>110</v>
       </c>
       <c r="B112" t="inlineStr">
@@ -3570,11 +3558,11 @@
         <v>1328.333333333334</v>
       </c>
       <c r="H112" t="n">
-        <v>-0.0498334057656092</v>
+        <v>-0.04983340576560924</v>
       </c>
     </row>
     <row r="113">
-      <c r="A113" s="1" t="n">
+      <c r="A113" t="n">
         <v>111</v>
       </c>
       <c r="B113" t="inlineStr">
@@ -3602,7 +3590,7 @@
       </c>
     </row>
     <row r="114">
-      <c r="A114" s="1" t="n">
+      <c r="A114" t="n">
         <v>112</v>
       </c>
       <c r="B114" t="inlineStr">
@@ -3626,11 +3614,11 @@
         <v>1156.246666666667</v>
       </c>
       <c r="H114" t="n">
-        <v>-0.2382595854427238</v>
+        <v>-0.2382595854427239</v>
       </c>
     </row>
     <row r="115">
-      <c r="A115" s="1" t="n">
+      <c r="A115" t="n">
         <v>113</v>
       </c>
       <c r="B115" t="inlineStr">
@@ -3654,11 +3642,11 @@
         <v>1291.846666666667</v>
       </c>
       <c r="H115" t="n">
-        <v>0.0542470272960267</v>
+        <v>0.05424702729602671</v>
       </c>
     </row>
     <row r="116">
-      <c r="A116" s="1" t="n">
+      <c r="A116" t="n">
         <v>114</v>
       </c>
       <c r="B116" t="inlineStr">
@@ -3682,11 +3670,11 @@
         <v>1281.120000000001</v>
       </c>
       <c r="H116" t="n">
-        <v>0.1167046046086128</v>
+        <v>0.1167046046086129</v>
       </c>
     </row>
     <row r="117">
-      <c r="A117" s="1" t="n">
+      <c r="A117" t="n">
         <v>115</v>
       </c>
       <c r="B117" t="inlineStr">
@@ -3710,11 +3698,11 @@
         <v>1626.433333333334</v>
       </c>
       <c r="H117" t="n">
-        <v>0.2948783104830756</v>
+        <v>0.2948783104830757</v>
       </c>
     </row>
     <row r="118">
-      <c r="A118" s="1" t="n">
+      <c r="A118" t="n">
         <v>116</v>
       </c>
       <c r="B118" t="inlineStr">
@@ -3735,14 +3723,14 @@
         <v>2263.833333333333</v>
       </c>
       <c r="G118" t="n">
-        <v>1838.573333333333</v>
+        <v>1838.573333333334</v>
       </c>
       <c r="H118" t="n">
         <v>-0.2254228844196244</v>
       </c>
     </row>
     <row r="119">
-      <c r="A119" s="1" t="n">
+      <c r="A119" t="n">
         <v>117</v>
       </c>
       <c r="B119" t="inlineStr">
@@ -3763,14 +3751,14 @@
         <v>2430.16129032258</v>
       </c>
       <c r="G119" t="n">
-        <v>1840.65</v>
+        <v>1840.650000000001</v>
       </c>
       <c r="H119" t="n">
-        <v>0.0422587405087135</v>
+        <v>0.04225874050871359</v>
       </c>
     </row>
     <row r="120">
-      <c r="A120" s="1" t="n">
+      <c r="A120" t="n">
         <v>118</v>
       </c>
       <c r="B120" t="inlineStr">
@@ -3791,14 +3779,14 @@
         <v>2531.6</v>
       </c>
       <c r="G120" t="n">
-        <v>1810.366666666668</v>
+        <v>1810.366666666667</v>
       </c>
       <c r="H120" t="n">
-        <v>0.0124202071694645</v>
+        <v>0.01242020716946457</v>
       </c>
     </row>
     <row r="121">
-      <c r="A121" s="1" t="n">
+      <c r="A121" t="n">
         <v>119</v>
       </c>
       <c r="B121" t="inlineStr">
@@ -3822,11 +3810,11 @@
         <v>1660.246666666667</v>
       </c>
       <c r="H121" t="n">
-        <v>0.0230123362515479</v>
+        <v>0.02301233625154797</v>
       </c>
     </row>
     <row r="122">
-      <c r="A122" s="1" t="n">
+      <c r="A122" t="n">
         <v>120</v>
       </c>
       <c r="B122" t="inlineStr">
@@ -3850,11 +3838,11 @@
         <v>1519.036666666667</v>
       </c>
       <c r="H122" t="n">
-        <v>-0.1060034539102333</v>
+        <v>-0.1060034539102334</v>
       </c>
     </row>
     <row r="123">
-      <c r="A123" s="1" t="n">
+      <c r="A123" t="n">
         <v>121</v>
       </c>
       <c r="B123" t="inlineStr">
@@ -3878,11 +3866,11 @@
         <v>1180.200000000001</v>
       </c>
       <c r="H123" t="n">
-        <v>-0.0465907892749567</v>
+        <v>-0.04659078927495675</v>
       </c>
     </row>
     <row r="124">
-      <c r="A124" s="1" t="n">
+      <c r="A124" t="n">
         <v>122</v>
       </c>
       <c r="B124" t="inlineStr">
@@ -3910,7 +3898,7 @@
       </c>
     </row>
     <row r="125">
-      <c r="A125" s="1" t="n">
+      <c r="A125" t="n">
         <v>123</v>
       </c>
       <c r="B125" t="inlineStr">
@@ -3934,11 +3922,11 @@
         <v>1442.330000000001</v>
       </c>
       <c r="H125" t="n">
-        <v>-0.0708237463575456</v>
+        <v>-0.07082374635754562</v>
       </c>
     </row>
     <row r="126">
-      <c r="A126" s="1" t="n">
+      <c r="A126" t="n">
         <v>124</v>
       </c>
       <c r="B126" t="inlineStr">
@@ -3962,11 +3950,11 @@
         <v>1606.400000000001</v>
       </c>
       <c r="H126" t="n">
-        <v>0.0589508985879332</v>
+        <v>0.05895089858793323</v>
       </c>
     </row>
     <row r="127">
-      <c r="A127" s="1" t="n">
+      <c r="A127" t="n">
         <v>125</v>
       </c>
       <c r="B127" t="inlineStr">
@@ -3984,17 +3972,17 @@
         <v>15024</v>
       </c>
       <c r="F127" t="n">
-        <v>1949.566666666666</v>
+        <v>1949.566666666667</v>
       </c>
       <c r="G127" t="n">
         <v>1367.743333333334</v>
       </c>
       <c r="H127" t="n">
-        <v>-0.2259911609905289</v>
+        <v>-0.225991160990529</v>
       </c>
     </row>
     <row r="128">
-      <c r="A128" s="1" t="n">
+      <c r="A128" t="n">
         <v>126</v>
       </c>
       <c r="B128" t="inlineStr">
@@ -4015,14 +4003,14 @@
         <v>2600.129032258064</v>
       </c>
       <c r="G128" t="n">
-        <v>1487.616666666668</v>
+        <v>1487.616666666667</v>
       </c>
       <c r="H128" t="n">
-        <v>0.1575017913147662</v>
+        <v>0.1575017913147663</v>
       </c>
     </row>
     <row r="129">
-      <c r="A129" s="1" t="n">
+      <c r="A129" t="n">
         <v>127</v>
       </c>
       <c r="B129" t="inlineStr">
@@ -4046,11 +4034,11 @@
         <v>1521.166666666667</v>
       </c>
       <c r="H129" t="n">
-        <v>-0.0650764076626859</v>
+        <v>-0.06507640766268596</v>
       </c>
     </row>
     <row r="130">
-      <c r="A130" s="1" t="n">
+      <c r="A130" t="n">
         <v>128</v>
       </c>
       <c r="B130" t="inlineStr">
@@ -4074,11 +4062,11 @@
         <v>1528.760000000001</v>
       </c>
       <c r="H130" t="n">
-        <v>0.0904826789721353</v>
+        <v>0.09048267897213536</v>
       </c>
     </row>
     <row r="131">
-      <c r="A131" s="1" t="n">
+      <c r="A131" t="n">
         <v>129</v>
       </c>
       <c r="B131" t="inlineStr">
@@ -4106,7 +4094,7 @@
       </c>
     </row>
     <row r="132">
-      <c r="A132" s="1" t="n">
+      <c r="A132" t="n">
         <v>130</v>
       </c>
       <c r="B132" t="inlineStr">
@@ -4134,7 +4122,7 @@
       </c>
     </row>
     <row r="133">
-      <c r="A133" s="1" t="n">
+      <c r="A133" t="n">
         <v>131</v>
       </c>
       <c r="B133" t="inlineStr">
@@ -4158,11 +4146,11 @@
         <v>1248.550000000001</v>
       </c>
       <c r="H133" t="n">
-        <v>0.0077639222790517</v>
+        <v>0.00776392227905176</v>
       </c>
     </row>
     <row r="134">
-      <c r="A134" s="1" t="n">
+      <c r="A134" t="n">
         <v>132</v>
       </c>
       <c r="B134" t="inlineStr">
@@ -4186,11 +4174,11 @@
         <v>1447.556666666667</v>
       </c>
       <c r="H134" t="n">
-        <v>-0.0322407594950558</v>
+        <v>-0.03224075949505589</v>
       </c>
     </row>
     <row r="135">
-      <c r="A135" s="1" t="n">
+      <c r="A135" t="n">
         <v>133</v>
       </c>
       <c r="B135" t="inlineStr">
@@ -4218,7 +4206,7 @@
       </c>
     </row>
     <row r="136">
-      <c r="A136" s="1" t="n">
+      <c r="A136" t="n">
         <v>134</v>
       </c>
       <c r="B136" t="inlineStr">
@@ -4246,7 +4234,7 @@
       </c>
     </row>
     <row r="137">
-      <c r="A137" s="1" t="n">
+      <c r="A137" t="n">
         <v>135</v>
       </c>
       <c r="B137" t="inlineStr">
@@ -4270,11 +4258,11 @@
         <v>1831.906666666667</v>
       </c>
       <c r="H137" t="n">
-        <v>0.0553096440130238</v>
+        <v>0.05530964401302385</v>
       </c>
     </row>
     <row r="138">
-      <c r="A138" s="1" t="n">
+      <c r="A138" t="n">
         <v>136</v>
       </c>
       <c r="B138" t="inlineStr">
@@ -4298,11 +4286,11 @@
         <v>1804.383333333334</v>
       </c>
       <c r="H138" t="n">
-        <v>-0.0177099818714442</v>
+        <v>-0.01770998187144424</v>
       </c>
     </row>
     <row r="139">
-      <c r="A139" s="1" t="n">
+      <c r="A139" t="n">
         <v>137</v>
       </c>
       <c r="B139" t="inlineStr">
@@ -4326,11 +4314,11 @@
         <v>1431.963333333334</v>
       </c>
       <c r="H139" t="n">
-        <v>-0.3469132334085448</v>
+        <v>-0.3469132334085449</v>
       </c>
     </row>
     <row r="140">
-      <c r="A140" s="1" t="n">
+      <c r="A140" t="n">
         <v>138</v>
       </c>
       <c r="B140" t="inlineStr">
@@ -4358,7 +4346,7 @@
       </c>
     </row>
     <row r="141">
-      <c r="A141" s="1" t="n">
+      <c r="A141" t="n">
         <v>139</v>
       </c>
       <c r="B141" t="inlineStr">
@@ -4382,11 +4370,11 @@
         <v>1291.206666666667</v>
       </c>
       <c r="H141" t="n">
-        <v>0.2034395569765394</v>
+        <v>0.2034395569765395</v>
       </c>
     </row>
     <row r="142">
-      <c r="A142" s="1" t="n">
+      <c r="A142" t="n">
         <v>140</v>
       </c>
       <c r="B142" t="inlineStr">
@@ -4410,11 +4398,11 @@
         <v>1632.806666666667</v>
       </c>
       <c r="H142" t="n">
-        <v>-0.0544976924192839</v>
+        <v>-0.05449769241928393</v>
       </c>
     </row>
     <row r="143">
-      <c r="A143" s="1" t="n">
+      <c r="A143" t="n">
         <v>141</v>
       </c>
       <c r="B143" t="inlineStr">
@@ -4438,11 +4426,11 @@
         <v>1594.533333333334</v>
       </c>
       <c r="H143" t="n">
-        <v>-0.0463627028364185</v>
+        <v>-0.04636270283641852</v>
       </c>
     </row>
     <row r="144">
-      <c r="A144" s="1" t="n">
+      <c r="A144" t="n">
         <v>142</v>
       </c>
       <c r="B144" t="inlineStr">
@@ -4466,11 +4454,11 @@
         <v>1513.530000000001</v>
       </c>
       <c r="H144" t="n">
-        <v>0.0504069458083915</v>
+        <v>0.05040694580839156</v>
       </c>
     </row>
     <row r="145">
-      <c r="A145" s="1" t="n">
+      <c r="A145" t="n">
         <v>143</v>
       </c>
       <c r="B145" t="inlineStr">
@@ -4494,11 +4482,11 @@
         <v>1284.263333333334</v>
       </c>
       <c r="H145" t="n">
-        <v>-0.0082240786406629</v>
+        <v>-0.008224078640662991</v>
       </c>
     </row>
     <row r="146">
-      <c r="A146" s="1" t="n">
+      <c r="A146" t="n">
         <v>144</v>
       </c>
       <c r="B146" t="inlineStr">
@@ -4526,7 +4514,7 @@
       </c>
     </row>
     <row r="147">
-      <c r="A147" s="1" t="n">
+      <c r="A147" t="n">
         <v>145</v>
       </c>
       <c r="B147" t="inlineStr">
@@ -4554,7 +4542,7 @@
       </c>
     </row>
     <row r="148">
-      <c r="A148" s="1" t="n">
+      <c r="A148" t="n">
         <v>146</v>
       </c>
       <c r="B148" t="inlineStr">
@@ -4572,17 +4560,17 @@
         <v>15492</v>
       </c>
       <c r="F148" t="n">
-        <v>2841.290322580646</v>
+        <v>2841.290322580645</v>
       </c>
       <c r="G148" t="n">
         <v>1259.213333333334</v>
       </c>
       <c r="H148" t="n">
-        <v>0.0501787201236754</v>
+        <v>0.05017872012367541</v>
       </c>
     </row>
     <row r="149">
-      <c r="A149" s="1" t="n">
+      <c r="A149" t="n">
         <v>147</v>
       </c>
       <c r="B149" t="inlineStr">
@@ -4610,7 +4598,7 @@
       </c>
     </row>
     <row r="150">
-      <c r="A150" s="1" t="n">
+      <c r="A150" t="n">
         <v>148</v>
       </c>
       <c r="B150" t="inlineStr">
@@ -4638,7 +4626,7 @@
       </c>
     </row>
     <row r="151">
-      <c r="A151" s="1" t="n">
+      <c r="A151" t="n">
         <v>149</v>
       </c>
       <c r="B151" t="inlineStr">
@@ -4662,11 +4650,11 @@
         <v>1274.320000000001</v>
       </c>
       <c r="H151" t="n">
-        <v>0.0562516119356342</v>
+        <v>0.05625161193563422</v>
       </c>
     </row>
     <row r="152">
-      <c r="A152" s="1" t="n">
+      <c r="A152" t="n">
         <v>150</v>
       </c>
       <c r="B152" t="inlineStr">
@@ -4684,17 +4672,17 @@
         <v>15429</v>
       </c>
       <c r="F152" t="n">
-        <v>2986.290322580646</v>
+        <v>2986.290322580645</v>
       </c>
       <c r="G152" t="n">
         <v>1345.856666666667</v>
       </c>
       <c r="H152" t="n">
-        <v>-0.111951925547573</v>
+        <v>-0.1119519255475731</v>
       </c>
     </row>
     <row r="153">
-      <c r="A153" s="1" t="n">
+      <c r="A153" t="n">
         <v>151</v>
       </c>
       <c r="B153" t="inlineStr">
@@ -4712,17 +4700,17 @@
         <v>15566</v>
       </c>
       <c r="F153" t="n">
-        <v>2845.290322580646</v>
+        <v>2845.290322580645</v>
       </c>
       <c r="G153" t="n">
         <v>1455.923333333334</v>
       </c>
       <c r="H153" t="n">
-        <v>0.1150879810273399</v>
+        <v>0.11508798102734</v>
       </c>
     </row>
     <row r="154">
-      <c r="A154" s="1" t="n">
+      <c r="A154" t="n">
         <v>152</v>
       </c>
       <c r="B154" t="inlineStr">
@@ -4746,11 +4734,11 @@
         <v>1643.286666666668</v>
       </c>
       <c r="H154" t="n">
-        <v>-0.0666760058410836</v>
+        <v>-0.06667600584108369</v>
       </c>
     </row>
     <row r="155">
-      <c r="A155" s="1" t="n">
+      <c r="A155" t="n">
         <v>153</v>
       </c>
       <c r="B155" t="inlineStr">
@@ -4774,11 +4762,11 @@
         <v>1713.540000000001</v>
       </c>
       <c r="H155" t="n">
-        <v>0.2209902116601931</v>
+        <v>0.2209902116601932</v>
       </c>
     </row>
     <row r="156">
-      <c r="A156" s="1" t="n">
+      <c r="A156" t="n">
         <v>154</v>
       </c>
       <c r="B156" t="inlineStr">
@@ -4806,7 +4794,7 @@
       </c>
     </row>
     <row r="157">
-      <c r="A157" s="1" t="n">
+      <c r="A157" t="n">
         <v>155</v>
       </c>
       <c r="B157" t="inlineStr">
@@ -4827,14 +4815,14 @@
         <v>2300.83870967742</v>
       </c>
       <c r="G157" t="n">
-        <v>1338.16</v>
+        <v>1338.160000000001</v>
       </c>
       <c r="H157" t="n">
-        <v>0.0681744301143607</v>
+        <v>0.06817443011436075</v>
       </c>
     </row>
     <row r="158">
-      <c r="A158" s="1" t="n">
+      <c r="A158" t="n">
         <v>156</v>
       </c>
       <c r="B158" t="inlineStr">
@@ -4862,7 +4850,7 @@
       </c>
     </row>
     <row r="159">
-      <c r="A159" s="1" t="n">
+      <c r="A159" t="n">
         <v>157</v>
       </c>
       <c r="B159" t="inlineStr">
@@ -4886,11 +4874,11 @@
         <v>1327.096666666667</v>
       </c>
       <c r="H159" t="n">
-        <v>-0.2346612822507575</v>
+        <v>-0.2346612822507576</v>
       </c>
     </row>
     <row r="160">
-      <c r="A160" s="1" t="n">
+      <c r="A160" t="n">
         <v>158</v>
       </c>
       <c r="B160" t="inlineStr">
@@ -4914,11 +4902,11 @@
         <v>1252.996666666667</v>
       </c>
       <c r="H160" t="n">
-        <v>-0.0292079068592708</v>
+        <v>-0.02920790685927088</v>
       </c>
     </row>
     <row r="161">
-      <c r="A161" s="1" t="n">
+      <c r="A161" t="n">
         <v>159</v>
       </c>
       <c r="B161" t="inlineStr">
@@ -4946,7 +4934,7 @@
       </c>
     </row>
     <row r="162">
-      <c r="A162" s="1" t="n">
+      <c r="A162" t="n">
         <v>160</v>
       </c>
       <c r="B162" t="inlineStr">
@@ -4970,11 +4958,11 @@
         <v>1420.953333333334</v>
       </c>
       <c r="H162" t="n">
-        <v>0.0560809965144832</v>
+        <v>0.05608099651448328</v>
       </c>
     </row>
     <row r="163">
-      <c r="A163" s="1" t="n">
+      <c r="A163" t="n">
         <v>161</v>
       </c>
       <c r="B163" t="inlineStr">
@@ -4998,11 +4986,11 @@
         <v>1851.076666666667</v>
       </c>
       <c r="H163" t="n">
-        <v>0.0038533779928673</v>
+        <v>0.003853377992867335</v>
       </c>
     </row>
     <row r="164">
-      <c r="A164" s="1" t="n">
+      <c r="A164" t="n">
         <v>162</v>
       </c>
       <c r="B164" t="inlineStr">
@@ -5020,7 +5008,7 @@
         <v>15520</v>
       </c>
       <c r="F164" t="n">
-        <v>2432.290322580646</v>
+        <v>2432.290322580645</v>
       </c>
       <c r="G164" t="n">
         <v>1871.106666666667</v>
@@ -5030,7 +5018,7 @@
       </c>
     </row>
     <row r="165">
-      <c r="A165" s="1" t="n">
+      <c r="A165" t="n">
         <v>163</v>
       </c>
       <c r="B165" t="inlineStr">
@@ -5054,11 +5042,11 @@
         <v>1804.860000000001</v>
       </c>
       <c r="H165" t="n">
-        <v>-0.0519190799122737</v>
+        <v>-0.05191907991227374</v>
       </c>
     </row>
     <row r="166">
-      <c r="A166" s="1" t="n">
+      <c r="A166" t="n">
         <v>164</v>
       </c>
       <c r="B166" t="inlineStr">
@@ -5082,11 +5070,11 @@
         <v>1544.000000000001</v>
       </c>
       <c r="H166" t="n">
-        <v>-0.2031599743496229</v>
+        <v>-0.203159974349623</v>
       </c>
     </row>
     <row r="167">
-      <c r="A167" s="1" t="n">
+      <c r="A167" t="n">
         <v>165</v>
       </c>
       <c r="B167" t="inlineStr">
@@ -5103,7 +5091,7 @@
       <c r="E167" t="n">
         <v>15411</v>
       </c>
-      <c r="F167" s="2" t="n">
+      <c r="F167" s="1" t="n">
         <v>3161.096774193548</v>
       </c>
       <c r="G167" t="n">
@@ -5114,7 +5102,7 @@
       </c>
     </row>
     <row r="168">
-      <c r="A168" s="1" t="n">
+      <c r="A168" t="n">
         <v>166</v>
       </c>
       <c r="B168" t="inlineStr">
@@ -5138,11 +5126,11 @@
         <v>1217.253333333334</v>
       </c>
       <c r="H168" t="n">
-        <v>0.09352219106145999</v>
+        <v>0.09352219106146009</v>
       </c>
     </row>
     <row r="169">
-      <c r="A169" s="1" t="n">
+      <c r="A169" t="n">
         <v>167</v>
       </c>
       <c r="B169" t="inlineStr">
@@ -5163,14 +5151,14 @@
         <v>2775.741935483871</v>
       </c>
       <c r="G169" t="n">
-        <v>1095.41</v>
+        <v>1095.410000000001</v>
       </c>
       <c r="H169" t="n">
-        <v>-0.0020073396893431</v>
+        <v>-0.002007339689343191</v>
       </c>
     </row>
     <row r="170">
-      <c r="A170" s="1" t="n">
+      <c r="A170" t="n">
         <v>168</v>
       </c>
       <c r="B170" t="inlineStr">
@@ -5194,11 +5182,11 @@
         <v>1212.460000000001</v>
       </c>
       <c r="H170" t="n">
-        <v>-0.1012987498905164</v>
+        <v>-0.1012987498905165</v>
       </c>
     </row>
     <row r="171">
-      <c r="A171" s="1" t="n">
+      <c r="A171" t="n">
         <v>169</v>
       </c>
       <c r="B171" t="inlineStr">
@@ -5222,11 +5210,11 @@
         <v>1326.926666666667</v>
       </c>
       <c r="H171" t="n">
-        <v>-0.0431063195225065</v>
+        <v>-0.04310631952250654</v>
       </c>
     </row>
     <row r="172">
-      <c r="A172" s="1" t="n">
+      <c r="A172" t="n">
         <v>170</v>
       </c>
       <c r="B172" t="inlineStr">
@@ -5250,11 +5238,11 @@
         <v>1358.920000000001</v>
       </c>
       <c r="H172" t="n">
-        <v>-0.0449980800195128</v>
+        <v>-0.04499808001951289</v>
       </c>
     </row>
     <row r="173">
-      <c r="A173" s="1" t="n">
+      <c r="A173" t="n">
         <v>171</v>
       </c>
       <c r="B173" t="inlineStr">
@@ -5282,7 +5270,7 @@
       </c>
     </row>
     <row r="174">
-      <c r="A174" s="1" t="n">
+      <c r="A174" t="n">
         <v>172</v>
       </c>
       <c r="B174" t="inlineStr">
@@ -5310,7 +5298,7 @@
       </c>
     </row>
     <row r="175">
-      <c r="A175" s="1" t="n">
+      <c r="A175" t="n">
         <v>173</v>
       </c>
       <c r="B175" t="inlineStr">
@@ -5338,7 +5326,7 @@
       </c>
     </row>
     <row r="176">
-      <c r="A176" s="1" t="n">
+      <c r="A176" t="n">
         <v>174</v>
       </c>
       <c r="B176" t="inlineStr">
@@ -5362,11 +5350,11 @@
         <v>1320.843333333334</v>
       </c>
       <c r="H176" t="n">
-        <v>0.022034042581055</v>
+        <v>0.02203404258105501</v>
       </c>
     </row>
     <row r="177">
-      <c r="A177" s="1" t="n">
+      <c r="A177" t="n">
         <v>175</v>
       </c>
       <c r="B177" t="inlineStr">
@@ -5390,11 +5378,11 @@
         <v>1357.566666666667</v>
       </c>
       <c r="H177" t="n">
-        <v>0.08124326691356119</v>
+        <v>0.08124326691356121</v>
       </c>
     </row>
     <row r="178">
-      <c r="A178" s="1" t="n">
+      <c r="A178" t="n">
         <v>176</v>
       </c>
       <c r="B178" t="inlineStr">
@@ -5418,11 +5406,11 @@
         <v>1426.306666666667</v>
       </c>
       <c r="H178" t="n">
-        <v>0.0331069949033115</v>
+        <v>0.03310699490331159</v>
       </c>
     </row>
     <row r="179">
-      <c r="A179" s="1" t="n">
+      <c r="A179" t="n">
         <v>177</v>
       </c>
       <c r="B179" t="inlineStr">
@@ -5450,7 +5438,7 @@
       </c>
     </row>
     <row r="180">
-      <c r="A180" s="1" t="n">
+      <c r="A180" t="n">
         <v>178</v>
       </c>
       <c r="B180" t="inlineStr">
@@ -5458,7 +5446,7 @@
           <t>2034-11</t>
         </is>
       </c>
-      <c r="C180" s="2" t="n">
+      <c r="C180" s="1" t="n">
         <v>39065.76</v>
       </c>
       <c r="D180" t="n">
@@ -5478,7 +5466,7 @@
       </c>
     </row>
     <row r="181">
-      <c r="A181" s="1" t="n">
+      <c r="A181" t="n">
         <v>179</v>
       </c>
       <c r="B181" t="inlineStr">
@@ -5502,11 +5490,11 @@
         <v>1843.700000000001</v>
       </c>
       <c r="H181" t="n">
-        <v>-0.0980062847874968</v>
+        <v>-0.09800628478749684</v>
       </c>
     </row>
     <row r="182">
-      <c r="A182" s="1" t="n">
+      <c r="A182" t="n">
         <v>180</v>
       </c>
       <c r="B182" t="inlineStr">
@@ -5530,11 +5518,11 @@
         <v>1857.526666666667</v>
       </c>
       <c r="H182" t="n">
-        <v>-0.1085808212771379</v>
+        <v>-0.108580821277138</v>
       </c>
     </row>
     <row r="183">
-      <c r="A183" s="1" t="n">
+      <c r="A183" t="n">
         <v>181</v>
       </c>
       <c r="B183" t="inlineStr">
@@ -5558,11 +5546,11 @@
         <v>1449.166666666667</v>
       </c>
       <c r="H183" t="n">
-        <v>0.0289510044252014</v>
+        <v>0.02895100442520149</v>
       </c>
     </row>
     <row r="184">
-      <c r="A184" s="1" t="n">
+      <c r="A184" t="n">
         <v>182</v>
       </c>
       <c r="B184" t="inlineStr">
@@ -5586,11 +5574,11 @@
         <v>1482.186666666667</v>
       </c>
       <c r="H184" t="n">
-        <v>-0.1220985025547348</v>
+        <v>-0.1220985025547349</v>
       </c>
     </row>
     <row r="185">
-      <c r="A185" s="1" t="n">
+      <c r="A185" t="n">
         <v>183</v>
       </c>
       <c r="B185" t="inlineStr">
@@ -5618,7 +5606,7 @@
       </c>
     </row>
     <row r="186">
-      <c r="A186" s="1" t="n">
+      <c r="A186" t="n">
         <v>184</v>
       </c>
       <c r="B186" t="inlineStr">
@@ -5646,7 +5634,7 @@
       </c>
     </row>
     <row r="187">
-      <c r="A187" s="1" t="n">
+      <c r="A187" t="n">
         <v>185</v>
       </c>
       <c r="B187" t="inlineStr">
@@ -5670,11 +5658,11 @@
         <v>1442.390000000001</v>
       </c>
       <c r="H187" t="n">
-        <v>0.0901354347390865</v>
+        <v>0.09013543473908658</v>
       </c>
     </row>
     <row r="188">
-      <c r="A188" s="1" t="n">
+      <c r="A188" t="n">
         <v>186</v>
       </c>
       <c r="B188" t="inlineStr">
@@ -5698,11 +5686,11 @@
         <v>1415.120000000001</v>
       </c>
       <c r="H188" t="n">
-        <v>-0.0209450609956374</v>
+        <v>-0.02094506099563742</v>
       </c>
     </row>
     <row r="189">
-      <c r="A189" s="1" t="n">
+      <c r="A189" t="n">
         <v>187</v>
       </c>
       <c r="B189" t="inlineStr">
@@ -5726,11 +5714,11 @@
         <v>1253.923333333334</v>
       </c>
       <c r="H189" t="n">
-        <v>-0.2320616281728392</v>
+        <v>-0.2320616281728393</v>
       </c>
     </row>
     <row r="190">
-      <c r="A190" s="1" t="n">
+      <c r="A190" t="n">
         <v>188</v>
       </c>
       <c r="B190" t="inlineStr">
@@ -5753,12 +5741,12 @@
       <c r="G190" t="n">
         <v>1494.936666666667</v>
       </c>
-      <c r="H190" s="2" t="n">
+      <c r="H190" s="1" t="n">
         <v>0.6039519383104996</v>
       </c>
     </row>
     <row r="191">
-      <c r="A191" s="1" t="n">
+      <c r="A191" t="n">
         <v>189</v>
       </c>
       <c r="B191" t="inlineStr">
@@ -5786,7 +5774,7 @@
       </c>
     </row>
     <row r="192">
-      <c r="A192" s="1" t="n">
+      <c r="A192" t="n">
         <v>190</v>
       </c>
       <c r="B192" t="inlineStr">
@@ -5810,11 +5798,11 @@
         <v>1501.906666666667</v>
       </c>
       <c r="H192" t="n">
-        <v>0.0572342852807992</v>
+        <v>0.05723428528079921</v>
       </c>
     </row>
     <row r="193">
-      <c r="A193" s="1" t="n">
+      <c r="A193" t="n">
         <v>191</v>
       </c>
       <c r="B193" t="inlineStr">
@@ -5838,11 +5826,11 @@
         <v>1252.646666666667</v>
       </c>
       <c r="H193" t="n">
-        <v>0.0293978442247839</v>
+        <v>0.02939784422478398</v>
       </c>
     </row>
     <row r="194">
-      <c r="A194" s="1" t="n">
+      <c r="A194" t="n">
         <v>192</v>
       </c>
       <c r="B194" t="inlineStr">
@@ -5870,7 +5858,7 @@
       </c>
     </row>
     <row r="195">
-      <c r="A195" s="1" t="n">
+      <c r="A195" t="n">
         <v>193</v>
       </c>
       <c r="B195" t="inlineStr">
@@ -5898,7 +5886,7 @@
       </c>
     </row>
     <row r="196">
-      <c r="A196" s="1" t="n">
+      <c r="A196" t="n">
         <v>194</v>
       </c>
       <c r="B196" t="inlineStr">
@@ -5926,7 +5914,7 @@
       </c>
     </row>
     <row r="197">
-      <c r="A197" s="1" t="n">
+      <c r="A197" t="n">
         <v>195</v>
       </c>
       <c r="B197" t="inlineStr">
@@ -5950,11 +5938,11 @@
         <v>1432.740000000001</v>
       </c>
       <c r="H197" t="n">
-        <v>0.0108657968204923</v>
+        <v>0.01086579682049238</v>
       </c>
     </row>
     <row r="198">
-      <c r="A198" s="1" t="n">
+      <c r="A198" t="n">
         <v>196</v>
       </c>
       <c r="B198" t="inlineStr">
@@ -5982,7 +5970,7 @@
       </c>
     </row>
     <row r="199">
-      <c r="A199" s="1" t="n">
+      <c r="A199" t="n">
         <v>197</v>
       </c>
       <c r="B199" t="inlineStr">
@@ -6010,7 +5998,7 @@
       </c>
     </row>
     <row r="200">
-      <c r="A200" s="1" t="n">
+      <c r="A200" t="n">
         <v>198</v>
       </c>
       <c r="B200" t="inlineStr">
@@ -6038,7 +6026,7 @@
       </c>
     </row>
     <row r="201">
-      <c r="A201" s="1" t="n">
+      <c r="A201" t="n">
         <v>199</v>
       </c>
       <c r="B201" t="inlineStr">
@@ -6062,11 +6050,11 @@
         <v>1595.796666666667</v>
       </c>
       <c r="H201" t="n">
-        <v>0.0553922029285136</v>
+        <v>0.05539220292851366</v>
       </c>
     </row>
     <row r="202">
-      <c r="A202" s="1" t="n">
+      <c r="A202" t="n">
         <v>200</v>
       </c>
       <c r="B202" t="inlineStr">
@@ -6090,11 +6078,11 @@
         <v>1382.203333333334</v>
       </c>
       <c r="H202" t="n">
-        <v>-0.0794504727302468</v>
+        <v>-0.07945047273024686</v>
       </c>
     </row>
     <row r="203">
-      <c r="A203" s="1" t="n">
+      <c r="A203" t="n">
         <v>201</v>
       </c>
       <c r="B203" t="inlineStr">
@@ -6118,11 +6106,11 @@
         <v>1328.853333333334</v>
       </c>
       <c r="H203" t="n">
-        <v>-0.0201844045364217</v>
+        <v>-0.02018440453642179</v>
       </c>
     </row>
     <row r="204">
-      <c r="A204" s="1" t="n">
+      <c r="A204" t="n">
         <v>202</v>
       </c>
       <c r="B204" t="inlineStr">
@@ -6143,14 +6131,14 @@
         <v>2574.5</v>
       </c>
       <c r="G204" t="n">
-        <v>1581.616666666668</v>
+        <v>1581.616666666667</v>
       </c>
       <c r="H204" t="n">
         <v>0.1712359795409248</v>
       </c>
     </row>
     <row r="205">
-      <c r="A205" s="1" t="n">
+      <c r="A205" t="n">
         <v>203</v>
       </c>
       <c r="B205" t="inlineStr">
@@ -6178,7 +6166,7 @@
       </c>
     </row>
     <row r="206">
-      <c r="A206" s="1" t="n">
+      <c r="A206" t="n">
         <v>204</v>
       </c>
       <c r="B206" t="inlineStr">
@@ -6206,7 +6194,7 @@
       </c>
     </row>
     <row r="207">
-      <c r="A207" s="1" t="n">
+      <c r="A207" t="n">
         <v>205</v>
       </c>
       <c r="B207" t="inlineStr">
@@ -6230,11 +6218,11 @@
         <v>1201.803333333334</v>
       </c>
       <c r="H207" t="n">
-        <v>-0.1979977738248671</v>
+        <v>-0.1979977738248672</v>
       </c>
     </row>
     <row r="208">
-      <c r="A208" s="1" t="n">
+      <c r="A208" t="n">
         <v>206</v>
       </c>
       <c r="B208" t="inlineStr">
@@ -6248,7 +6236,7 @@
       <c r="D208" t="n">
         <v>1641.75</v>
       </c>
-      <c r="E208" s="2" t="n">
+      <c r="E208" s="1" t="n">
         <v>15835</v>
       </c>
       <c r="F208" t="n">
@@ -6262,7 +6250,7 @@
       </c>
     </row>
     <row r="209">
-      <c r="A209" s="1" t="n">
+      <c r="A209" t="n">
         <v>207</v>
       </c>
       <c r="B209" t="inlineStr">
@@ -6286,11 +6274,11 @@
         <v>1255.976666666667</v>
       </c>
       <c r="H209" t="n">
-        <v>-0.0237050659264399</v>
+        <v>-0.02370506592643995</v>
       </c>
     </row>
     <row r="210">
-      <c r="A210" s="1" t="n">
+      <c r="A210" t="n">
         <v>208</v>
       </c>
       <c r="B210" t="inlineStr">
@@ -6314,11 +6302,11 @@
         <v>1199.526666666667</v>
       </c>
       <c r="H210" t="n">
-        <v>-0.0274099916053057</v>
+        <v>-0.02740999160530577</v>
       </c>
     </row>
     <row r="211">
-      <c r="A211" s="1" t="n">
+      <c r="A211" t="n">
         <v>209</v>
       </c>
       <c r="B211" t="inlineStr">
@@ -6342,11 +6330,11 @@
         <v>1087.690000000001</v>
       </c>
       <c r="H211" t="n">
-        <v>0.1202374953362963</v>
+        <v>0.1202374953362964</v>
       </c>
     </row>
     <row r="212">
-      <c r="A212" s="1" t="n">
+      <c r="A212" t="n">
         <v>210</v>
       </c>
       <c r="B212" t="inlineStr">
@@ -6364,17 +6352,17 @@
         <v>15439</v>
       </c>
       <c r="F212" t="n">
-        <v>2518.709677419354</v>
+        <v>2518.709677419355</v>
       </c>
       <c r="G212" t="n">
         <v>1134.836666666667</v>
       </c>
       <c r="H212" t="n">
-        <v>0.0059045614621104</v>
+        <v>0.005904561462110491</v>
       </c>
     </row>
     <row r="213">
-      <c r="A213" s="1" t="n">
+      <c r="A213" t="n">
         <v>211</v>
       </c>
       <c r="B213" t="inlineStr">
@@ -6398,11 +6386,11 @@
         <v>1013.110000000001</v>
       </c>
       <c r="H213" t="n">
-        <v>-0.0880722068348479</v>
+        <v>-0.08807220683484795</v>
       </c>
     </row>
     <row r="214">
-      <c r="A214" s="1" t="n">
+      <c r="A214" t="n">
         <v>212</v>
       </c>
       <c r="B214" t="inlineStr">
@@ -6426,11 +6414,11 @@
         <v>902.0266666666672</v>
       </c>
       <c r="H214" t="n">
-        <v>-0.0414361605471196</v>
+        <v>-0.04143616054711963</v>
       </c>
     </row>
     <row r="215">
-      <c r="A215" s="1" t="n">
+      <c r="A215" t="n">
         <v>213</v>
       </c>
       <c r="B215" t="inlineStr">
@@ -6451,14 +6439,14 @@
         <v>2323.41935483871</v>
       </c>
       <c r="G215" t="n">
-        <v>920.7066666666672</v>
+        <v>920.7066666666673</v>
       </c>
       <c r="H215" t="n">
-        <v>0.1098573742407031</v>
+        <v>0.1098573742407032</v>
       </c>
     </row>
     <row r="216">
-      <c r="A216" s="1" t="n">
+      <c r="A216" t="n">
         <v>214</v>
       </c>
       <c r="B216" t="inlineStr">
@@ -6482,11 +6470,11 @@
         <v>1080.310000000001</v>
       </c>
       <c r="H216" t="n">
-        <v>0.0335265780575428</v>
+        <v>0.03352657805754289</v>
       </c>
     </row>
     <row r="217">
-      <c r="A217" s="1" t="n">
+      <c r="A217" t="n">
         <v>215</v>
       </c>
       <c r="B217" t="inlineStr">
@@ -6504,17 +6492,17 @@
         <v>15583</v>
       </c>
       <c r="F217" t="n">
-        <v>2384.709677419354</v>
+        <v>2384.709677419355</v>
       </c>
       <c r="G217" t="n">
         <v>1538.503333333334</v>
       </c>
       <c r="H217" t="n">
-        <v>0.0975065475039278</v>
+        <v>0.09750654750392784</v>
       </c>
     </row>
     <row r="218">
-      <c r="A218" s="1" t="n">
+      <c r="A218" t="n">
         <v>216</v>
       </c>
       <c r="B218" t="inlineStr">
@@ -6538,11 +6526,11 @@
         <v>1805.553333333334</v>
       </c>
       <c r="H218" t="n">
-        <v>0.07546286882902969</v>
+        <v>0.07546286882902975</v>
       </c>
     </row>
     <row r="219">
-      <c r="A219" s="1" t="n">
+      <c r="A219" t="n">
         <v>217</v>
       </c>
       <c r="B219" t="inlineStr">
@@ -6570,7 +6558,7 @@
       </c>
     </row>
     <row r="220">
-      <c r="A220" s="1" t="n">
+      <c r="A220" t="n">
         <v>218</v>
       </c>
       <c r="B220" t="inlineStr">
@@ -6598,7 +6586,7 @@
       </c>
     </row>
     <row r="221">
-      <c r="A221" s="1" t="n">
+      <c r="A221" t="n">
         <v>219</v>
       </c>
       <c r="B221" t="inlineStr">
@@ -6626,7 +6614,7 @@
       </c>
     </row>
     <row r="222">
-      <c r="A222" s="1" t="n">
+      <c r="A222" t="n">
         <v>220</v>
       </c>
       <c r="B222" t="inlineStr">
@@ -6654,7 +6642,7 @@
       </c>
     </row>
     <row r="223">
-      <c r="A223" s="1" t="n">
+      <c r="A223" t="n">
         <v>221</v>
       </c>
       <c r="B223" t="inlineStr">
@@ -6678,11 +6666,11 @@
         <v>1800.946666666667</v>
       </c>
       <c r="H223" t="n">
-        <v>0.0825964331075852</v>
+        <v>0.08259643310758524</v>
       </c>
     </row>
     <row r="224">
-      <c r="A224" s="1" t="n">
+      <c r="A224" t="n">
         <v>222</v>
       </c>
       <c r="B224" t="inlineStr">
@@ -6706,11 +6694,11 @@
         <v>1770.353333333334</v>
       </c>
       <c r="H224" t="n">
-        <v>0.2900928338152448</v>
+        <v>0.2900928338152449</v>
       </c>
     </row>
     <row r="225">
-      <c r="A225" s="1" t="n">
+      <c r="A225" t="n">
         <v>223</v>
       </c>
       <c r="B225" t="inlineStr">
@@ -6738,7 +6726,7 @@
       </c>
     </row>
     <row r="226">
-      <c r="A226" s="1" t="n">
+      <c r="A226" t="n">
         <v>224</v>
       </c>
       <c r="B226" t="inlineStr">
@@ -6766,7 +6754,7 @@
       </c>
     </row>
     <row r="227">
-      <c r="A227" s="1" t="n">
+      <c r="A227" t="n">
         <v>225</v>
       </c>
       <c r="B227" t="inlineStr">
@@ -6790,11 +6778,11 @@
         <v>1324.966666666667</v>
       </c>
       <c r="H227" t="n">
-        <v>0.0680320815478736</v>
+        <v>0.06803208154787366</v>
       </c>
     </row>
     <row r="228">
-      <c r="A228" s="1" t="n">
+      <c r="A228" t="n">
         <v>226</v>
       </c>
       <c r="B228" t="inlineStr">
@@ -6818,11 +6806,11 @@
         <v>1437.373333333334</v>
       </c>
       <c r="H228" t="n">
-        <v>0.0475548283388755</v>
+        <v>0.04755482833887559</v>
       </c>
     </row>
     <row r="229">
-      <c r="A229" s="1" t="n">
+      <c r="A229" t="n">
         <v>227</v>
       </c>
       <c r="B229" t="inlineStr">
@@ -6846,11 +6834,11 @@
         <v>1404.333333333334</v>
       </c>
       <c r="H229" t="n">
-        <v>-0.07921870856019581</v>
+        <v>-0.07921870856019586</v>
       </c>
     </row>
     <row r="230">
-      <c r="A230" s="1" t="n">
+      <c r="A230" t="n">
         <v>228</v>
       </c>
       <c r="B230" t="inlineStr">
@@ -6874,11 +6862,11 @@
         <v>1398.360000000001</v>
       </c>
       <c r="H230" t="n">
-        <v>0.1439443074314363</v>
+        <v>0.1439443074314364</v>
       </c>
     </row>
     <row r="231">
-      <c r="A231" s="1" t="n">
+      <c r="A231" t="n">
         <v>229</v>
       </c>
       <c r="B231" t="inlineStr">
@@ -6906,7 +6894,7 @@
       </c>
     </row>
     <row r="232">
-      <c r="A232" s="1" t="n">
+      <c r="A232" t="n">
         <v>230</v>
       </c>
       <c r="B232" t="inlineStr">
@@ -6930,11 +6918,11 @@
         <v>1337.700000000001</v>
       </c>
       <c r="H232" t="n">
-        <v>-0.0029508394977123</v>
+        <v>-0.002950839497712354</v>
       </c>
     </row>
     <row r="233">
-      <c r="A233" s="1" t="n">
+      <c r="A233" t="n">
         <v>231</v>
       </c>
       <c r="B233" t="inlineStr">
@@ -6958,11 +6946,11 @@
         <v>1268.736666666667</v>
       </c>
       <c r="H233" t="n">
-        <v>0.0116276804587704</v>
+        <v>0.0116276804587705</v>
       </c>
     </row>
     <row r="234">
-      <c r="A234" s="1" t="n">
+      <c r="A234" t="n">
         <v>232</v>
       </c>
       <c r="B234" t="inlineStr">
@@ -6986,11 +6974,11 @@
         <v>1269.783333333334</v>
       </c>
       <c r="H234" t="n">
-        <v>0.2000996985064844</v>
+        <v>0.2000996985064845</v>
       </c>
     </row>
     <row r="235">
-      <c r="A235" s="1" t="n">
+      <c r="A235" t="n">
         <v>233</v>
       </c>
       <c r="B235" t="inlineStr">
@@ -7018,7 +7006,7 @@
       </c>
     </row>
     <row r="236">
-      <c r="A236" s="1" t="n">
+      <c r="A236" t="n">
         <v>234</v>
       </c>
       <c r="B236" t="inlineStr">
@@ -7046,7 +7034,7 @@
       </c>
     </row>
     <row r="237">
-      <c r="A237" s="1" t="n">
+      <c r="A237" t="n">
         <v>235</v>
       </c>
       <c r="B237" t="inlineStr">
@@ -7074,7 +7062,7 @@
       </c>
     </row>
     <row r="238">
-      <c r="A238" s="1" t="n">
+      <c r="A238" t="n">
         <v>236</v>
       </c>
       <c r="B238" t="inlineStr">
@@ -7102,7 +7090,7 @@
       </c>
     </row>
     <row r="239">
-      <c r="A239" s="1" t="n">
+      <c r="A239" t="n">
         <v>237</v>
       </c>
       <c r="B239" t="inlineStr">
@@ -7130,7 +7118,7 @@
       </c>
     </row>
     <row r="240">
-      <c r="A240" s="1" t="n">
+      <c r="A240" t="n">
         <v>238</v>
       </c>
       <c r="B240" t="inlineStr">
@@ -7154,11 +7142,11 @@
         <v>1592.786666666667</v>
       </c>
       <c r="H240" t="n">
-        <v>0.0008963310822935</v>
+        <v>0.0008963310822935888</v>
       </c>
     </row>
     <row r="241">
-      <c r="A241" s="1" t="n">
+      <c r="A241" t="n">
         <v>239</v>
       </c>
       <c r="B241" t="inlineStr">
@@ -7182,11 +7170,11 @@
         <v>1390.766666666667</v>
       </c>
       <c r="H241" t="n">
-        <v>-0.0802596915732586</v>
+        <v>-0.08025969157325863</v>
       </c>
     </row>
     <row r="242">
-      <c r="A242" s="1" t="n">
+      <c r="A242" t="n">
         <v>240</v>
       </c>
       <c r="B242" t="inlineStr">
@@ -7214,7 +7202,7 @@
       </c>
     </row>
     <row r="243">
-      <c r="A243" s="1" t="n">
+      <c r="A243" t="n">
         <v>241</v>
       </c>
       <c r="B243" t="inlineStr">
@@ -7242,7 +7230,7 @@
       </c>
     </row>
     <row r="244">
-      <c r="A244" s="1" t="n">
+      <c r="A244" t="n">
         <v>242</v>
       </c>
       <c r="B244" t="inlineStr">
@@ -7266,11 +7254,11 @@
         <v>1701.356666666667</v>
       </c>
       <c r="H244" t="n">
-        <v>-0.0106235869780748</v>
+        <v>-0.01062358697807486</v>
       </c>
     </row>
     <row r="245">
-      <c r="A245" s="1" t="n">
+      <c r="A245" t="n">
         <v>243</v>
       </c>
       <c r="B245" t="inlineStr">
@@ -7298,7 +7286,7 @@
       </c>
     </row>
     <row r="246">
-      <c r="A246" s="1" t="n">
+      <c r="A246" t="n">
         <v>244</v>
       </c>
       <c r="B246" t="inlineStr">
@@ -7326,7 +7314,7 @@
       </c>
     </row>
     <row r="247">
-      <c r="A247" s="1" t="n">
+      <c r="A247" t="n">
         <v>245</v>
       </c>
       <c r="B247" t="inlineStr">
@@ -7350,11 +7338,11 @@
         <v>1816.263333333334</v>
       </c>
       <c r="H247" t="n">
-        <v>-0.0380214271865212</v>
+        <v>-0.03802142718652124</v>
       </c>
     </row>
     <row r="248">
-      <c r="A248" s="1" t="n">
+      <c r="A248" t="n">
         <v>246</v>
       </c>
       <c r="B248" t="inlineStr">
@@ -7378,11 +7366,11 @@
         <v>1842.213333333334</v>
       </c>
       <c r="H248" t="n">
-        <v>-0.0800154583512078</v>
+        <v>-0.08001545835120782</v>
       </c>
     </row>
     <row r="249">
-      <c r="A249" s="1" t="n">
+      <c r="A249" t="n">
         <v>247</v>
       </c>
       <c r="B249" t="inlineStr">
@@ -7406,11 +7394,11 @@
         <v>1598.506666666667</v>
       </c>
       <c r="H249" t="n">
-        <v>-0.0154082962337657</v>
+        <v>-0.01540829623376572</v>
       </c>
     </row>
     <row r="250">
-      <c r="A250" s="1" t="n">
+      <c r="A250" t="n">
         <v>248</v>
       </c>
       <c r="B250" t="inlineStr">
@@ -7434,11 +7422,11 @@
         <v>1653.526666666667</v>
       </c>
       <c r="H250" t="n">
-        <v>-0.08842060782937471</v>
+        <v>-0.08842060782937478</v>
       </c>
     </row>
     <row r="251">
-      <c r="A251" s="1" t="n">
+      <c r="A251" t="n">
         <v>249</v>
       </c>
       <c r="B251" t="inlineStr">
@@ -7466,7 +7454,7 @@
       </c>
     </row>
     <row r="252">
-      <c r="A252" s="1" t="n">
+      <c r="A252" t="n">
         <v>250</v>
       </c>
       <c r="B252" t="inlineStr">
@@ -7490,11 +7478,11 @@
         <v>1611.590000000001</v>
       </c>
       <c r="H252" t="n">
-        <v>-0.1149489431707254</v>
+        <v>-0.1149489431707255</v>
       </c>
     </row>
     <row r="253">
-      <c r="A253" s="1" t="n">
+      <c r="A253" t="n">
         <v>251</v>
       </c>
       <c r="B253" t="inlineStr">
@@ -7518,11 +7506,11 @@
         <v>1462.623333333334</v>
       </c>
       <c r="H253" t="n">
-        <v>-0.07267001161948421</v>
+        <v>-0.07267001161948428</v>
       </c>
     </row>
     <row r="254">
-      <c r="A254" s="1" t="n">
+      <c r="A254" t="n">
         <v>252</v>
       </c>
       <c r="B254" t="inlineStr">
@@ -7550,7 +7538,7 @@
       </c>
     </row>
     <row r="255">
-      <c r="A255" s="1" t="n">
+      <c r="A255" t="n">
         <v>253</v>
       </c>
       <c r="B255" t="inlineStr">
@@ -7574,11 +7562,11 @@
         <v>1347.976666666667</v>
       </c>
       <c r="H255" t="n">
-        <v>-0.0983759916063953</v>
+        <v>-0.09837599160639532</v>
       </c>
     </row>
     <row r="256">
-      <c r="A256" s="1" t="n">
+      <c r="A256" t="n">
         <v>254</v>
       </c>
       <c r="B256" t="inlineStr">
@@ -7602,11 +7590,11 @@
         <v>1354.246666666667</v>
       </c>
       <c r="H256" t="n">
-        <v>-0.0745608896472921</v>
+        <v>-0.07456088964729213</v>
       </c>
     </row>
     <row r="257">
-      <c r="A257" s="1" t="n">
+      <c r="A257" t="n">
         <v>255</v>
       </c>
       <c r="B257" t="inlineStr">
@@ -7630,11 +7618,11 @@
         <v>1306.090000000001</v>
       </c>
       <c r="H257" t="n">
-        <v>0.1885529194661361</v>
+        <v>0.1885529194661362</v>
       </c>
     </row>
     <row r="258">
-      <c r="A258" s="1" t="n">
+      <c r="A258" t="n">
         <v>256</v>
       </c>
       <c r="B258" t="inlineStr">
@@ -7658,11 +7646,11 @@
         <v>1367.353333333334</v>
       </c>
       <c r="H258" t="n">
-        <v>-0.188607119461681</v>
+        <v>-0.1886071194616811</v>
       </c>
     </row>
     <row r="259">
-      <c r="A259" s="1" t="n">
+      <c r="A259" t="n">
         <v>257</v>
       </c>
       <c r="B259" t="inlineStr">
@@ -7690,7 +7678,7 @@
       </c>
     </row>
     <row r="260">
-      <c r="A260" s="1" t="n">
+      <c r="A260" t="n">
         <v>258</v>
       </c>
       <c r="B260" t="inlineStr">
@@ -7714,11 +7702,11 @@
         <v>1559.453333333334</v>
       </c>
       <c r="H260" t="n">
-        <v>0.046845831366963</v>
+        <v>0.04684583136696308</v>
       </c>
     </row>
     <row r="261">
-      <c r="A261" s="1" t="n">
+      <c r="A261" t="n">
         <v>259</v>
       </c>
       <c r="B261" t="inlineStr">
@@ -7742,11 +7730,11 @@
         <v>1657.876666666667</v>
       </c>
       <c r="H261" t="n">
-        <v>0.0296275310887781</v>
+        <v>0.02962753108877814</v>
       </c>
     </row>
     <row r="262">
-      <c r="A262" s="1" t="n">
+      <c r="A262" t="n">
         <v>260</v>
       </c>
       <c r="B262" t="inlineStr">
@@ -7770,11 +7758,11 @@
         <v>1644.736666666667</v>
       </c>
       <c r="H262" t="n">
-        <v>-0.0117282716236156</v>
+        <v>-0.01172827162361567</v>
       </c>
     </row>
     <row r="263">
-      <c r="A263" s="1" t="n">
+      <c r="A263" t="n">
         <v>261</v>
       </c>
       <c r="B263" t="inlineStr">
@@ -7792,17 +7780,17 @@
         <v>15619</v>
       </c>
       <c r="F263" t="n">
-        <v>2561.709677419354</v>
+        <v>2561.709677419355</v>
       </c>
       <c r="G263" t="n">
         <v>1580.696666666667</v>
       </c>
       <c r="H263" t="n">
-        <v>-0.042866758931692</v>
+        <v>-0.04286675893169201</v>
       </c>
     </row>
     <row r="264">
-      <c r="A264" s="1" t="n">
+      <c r="A264" t="n">
         <v>262</v>
       </c>
       <c r="B264" t="inlineStr">
@@ -7826,11 +7814,11 @@
         <v>1495.59</v>
       </c>
       <c r="H264" t="n">
-        <v>-0.0333081970790911</v>
+        <v>-0.03330819707909116</v>
       </c>
     </row>
     <row r="265">
-      <c r="A265" s="1" t="n">
+      <c r="A265" t="n">
         <v>263</v>
       </c>
       <c r="B265" t="inlineStr">
@@ -7854,11 +7842,11 @@
         <v>1446.693333333334</v>
       </c>
       <c r="H265" t="n">
-        <v>0.1257702563045015</v>
+        <v>0.1257702563045016</v>
       </c>
     </row>
     <row r="266">
-      <c r="A266" s="1" t="n">
+      <c r="A266" t="n">
         <v>264</v>
       </c>
       <c r="B266" t="inlineStr">
@@ -7886,7 +7874,7 @@
       </c>
     </row>
     <row r="267">
-      <c r="A267" s="1" t="n">
+      <c r="A267" t="n">
         <v>265</v>
       </c>
       <c r="B267" t="inlineStr">
@@ -7914,7 +7902,7 @@
       </c>
     </row>
     <row r="268">
-      <c r="A268" s="1" t="n">
+      <c r="A268" t="n">
         <v>266</v>
       </c>
       <c r="B268" t="inlineStr">
@@ -7942,7 +7930,7 @@
       </c>
     </row>
     <row r="269">
-      <c r="A269" s="1" t="n">
+      <c r="A269" t="n">
         <v>267</v>
       </c>
       <c r="B269" t="inlineStr">
@@ -7970,7 +7958,7 @@
       </c>
     </row>
     <row r="270">
-      <c r="A270" s="1" t="n">
+      <c r="A270" t="n">
         <v>268</v>
       </c>
       <c r="B270" t="inlineStr">
@@ -7998,7 +7986,7 @@
       </c>
     </row>
     <row r="271">
-      <c r="A271" s="1" t="n">
+      <c r="A271" t="n">
         <v>269</v>
       </c>
       <c r="B271" t="inlineStr">
@@ -8022,11 +8010,11 @@
         <v>1191.093333333334</v>
       </c>
       <c r="H271" t="n">
-        <v>0.0576397106441703</v>
+        <v>0.05763971064417039</v>
       </c>
     </row>
     <row r="272">
-      <c r="A272" s="1" t="n">
+      <c r="A272" t="n">
         <v>270</v>
       </c>
       <c r="B272" t="inlineStr">
@@ -8050,11 +8038,11 @@
         <v>1286.916666666667</v>
       </c>
       <c r="H272" t="n">
-        <v>0.009240914295674999</v>
+        <v>0.009240914295675084</v>
       </c>
     </row>
     <row r="273">
-      <c r="A273" s="1" t="n">
+      <c r="A273" t="n">
         <v>271</v>
       </c>
       <c r="B273" t="inlineStr">
@@ -8078,11 +8066,11 @@
         <v>1715.233333333334</v>
       </c>
       <c r="H273" t="n">
-        <v>0.0801000393937185</v>
+        <v>0.08010003939371857</v>
       </c>
     </row>
     <row r="274">
-      <c r="A274" s="1" t="n">
+      <c r="A274" t="n">
         <v>272</v>
       </c>
       <c r="B274" t="inlineStr">
@@ -8110,7 +8098,7 @@
       </c>
     </row>
     <row r="275">
-      <c r="A275" s="1" t="n">
+      <c r="A275" t="n">
         <v>273</v>
       </c>
       <c r="B275" t="inlineStr">
@@ -8134,11 +8122,11 @@
         <v>1847.236666666667</v>
       </c>
       <c r="H275" t="n">
-        <v>0.069849465607618</v>
+        <v>0.06984946560761807</v>
       </c>
     </row>
     <row r="276">
-      <c r="A276" s="1" t="n">
+      <c r="A276" t="n">
         <v>274</v>
       </c>
       <c r="B276" t="inlineStr">
@@ -8162,11 +8150,11 @@
         <v>1571.703333333334</v>
       </c>
       <c r="H276" t="n">
-        <v>-0.0336350212394941</v>
+        <v>-0.03363502123949413</v>
       </c>
     </row>
     <row r="277">
-      <c r="A277" s="1" t="n">
+      <c r="A277" t="n">
         <v>275</v>
       </c>
       <c r="B277" t="inlineStr">
@@ -8190,11 +8178,11 @@
         <v>1660.410000000001</v>
       </c>
       <c r="H277" t="n">
-        <v>0.0699644208546288</v>
+        <v>0.06996442085462884</v>
       </c>
     </row>
     <row r="278">
-      <c r="A278" s="1" t="n">
+      <c r="A278" t="n">
         <v>276</v>
       </c>
       <c r="B278" t="inlineStr">
@@ -8222,7 +8210,7 @@
       </c>
     </row>
     <row r="279">
-      <c r="A279" s="1" t="n">
+      <c r="A279" t="n">
         <v>277</v>
       </c>
       <c r="B279" t="inlineStr">
@@ -8246,11 +8234,11 @@
         <v>1410.873333333334</v>
       </c>
       <c r="H279" t="n">
-        <v>0.1331203443842878</v>
+        <v>0.1331203443842879</v>
       </c>
     </row>
     <row r="280">
-      <c r="A280" s="1" t="n">
+      <c r="A280" t="n">
         <v>278</v>
       </c>
       <c r="B280" t="inlineStr">
@@ -8268,7 +8256,7 @@
         <v>15387</v>
       </c>
       <c r="F280" t="n">
-        <v>2505.290322580646</v>
+        <v>2505.290322580645</v>
       </c>
       <c r="G280" t="n">
         <v>1525.456666666667</v>
@@ -8278,7 +8266,7 @@
       </c>
     </row>
     <row r="281">
-      <c r="A281" s="1" t="n">
+      <c r="A281" t="n">
         <v>279</v>
       </c>
       <c r="B281" t="inlineStr">
@@ -8302,11 +8290,11 @@
         <v>1566.813333333334</v>
       </c>
       <c r="H281" t="n">
-        <v>0.0853314331260199</v>
+        <v>0.08533143312601998</v>
       </c>
     </row>
     <row r="282">
-      <c r="A282" s="1" t="n">
+      <c r="A282" t="n">
         <v>280</v>
       </c>
       <c r="B282" t="inlineStr">
@@ -8330,11 +8318,11 @@
         <v>1835.013333333334</v>
       </c>
       <c r="H282" t="n">
-        <v>0.1380135101600907</v>
+        <v>0.1380135101600908</v>
       </c>
     </row>
     <row r="283">
-      <c r="A283" s="1" t="n">
+      <c r="A283" t="n">
         <v>281</v>
       </c>
       <c r="B283" t="inlineStr">
@@ -8358,11 +8346,11 @@
         <v>1850.920000000001</v>
       </c>
       <c r="H283" t="n">
-        <v>-0.1383111774852274</v>
+        <v>-0.1383111774852275</v>
       </c>
     </row>
     <row r="284">
-      <c r="A284" s="1" t="n">
+      <c r="A284" t="n">
         <v>282</v>
       </c>
       <c r="B284" t="inlineStr">
@@ -8386,11 +8374,11 @@
         <v>1816.243333333334</v>
       </c>
       <c r="H284" t="n">
-        <v>-0.1840499868178879</v>
+        <v>-0.184049986817888</v>
       </c>
     </row>
     <row r="285">
-      <c r="A285" s="1" t="n">
+      <c r="A285" t="n">
         <v>283</v>
       </c>
       <c r="B285" t="inlineStr">
@@ -8408,7 +8396,7 @@
         <v>15458</v>
       </c>
       <c r="F285" t="n">
-        <v>2745.290322580646</v>
+        <v>2745.290322580645</v>
       </c>
       <c r="G285" t="n">
         <v>1500.080000000001</v>
@@ -8418,7 +8406,7 @@
       </c>
     </row>
     <row r="286">
-      <c r="A286" s="1" t="n">
+      <c r="A286" t="n">
         <v>284</v>
       </c>
       <c r="B286" t="inlineStr">
@@ -8436,7 +8424,7 @@
         <v>14774</v>
       </c>
       <c r="F286" t="n">
-        <v>1894.933333333334</v>
+        <v>1894.933333333333</v>
       </c>
       <c r="G286" t="n">
         <v>1311.113333333334</v>
@@ -8446,7 +8434,7 @@
       </c>
     </row>
     <row r="287">
-      <c r="A287" s="1" t="n">
+      <c r="A287" t="n">
         <v>285</v>
       </c>
       <c r="B287" t="inlineStr">
@@ -8474,7 +8462,7 @@
       </c>
     </row>
     <row r="288">
-      <c r="A288" s="1" t="n">
+      <c r="A288" t="n">
         <v>286</v>
       </c>
       <c r="B288" t="inlineStr">
@@ -8498,11 +8486,11 @@
         <v>1583.700000000001</v>
       </c>
       <c r="H288" t="n">
-        <v>0.0681419663548166</v>
+        <v>0.06814196635481662</v>
       </c>
     </row>
     <row r="289">
-      <c r="A289" s="1" t="n">
+      <c r="A289" t="n">
         <v>287</v>
       </c>
       <c r="B289" t="inlineStr">
@@ -8530,7 +8518,7 @@
       </c>
     </row>
     <row r="290">
-      <c r="A290" s="1" t="n">
+      <c r="A290" t="n">
         <v>288</v>
       </c>
       <c r="B290" t="inlineStr">
@@ -8554,11 +8542,11 @@
         <v>1761.666666666667</v>
       </c>
       <c r="H290" t="n">
-        <v>0.0386276568134893</v>
+        <v>0.03862765681348934</v>
       </c>
     </row>
     <row r="291">
-      <c r="A291" s="1" t="n">
+      <c r="A291" t="n">
         <v>289</v>
       </c>
       <c r="B291" t="inlineStr">
@@ -8586,7 +8574,7 @@
       </c>
     </row>
     <row r="292">
-      <c r="A292" s="1" t="n">
+      <c r="A292" t="n">
         <v>290</v>
       </c>
       <c r="B292" t="inlineStr">
@@ -8610,11 +8598,11 @@
         <v>1291.24</v>
       </c>
       <c r="H292" t="n">
-        <v>0.2924450688801709</v>
+        <v>0.292445068880171</v>
       </c>
     </row>
     <row r="293">
-      <c r="A293" s="1" t="n">
+      <c r="A293" t="n">
         <v>291</v>
       </c>
       <c r="B293" t="inlineStr">
@@ -8642,7 +8630,7 @@
       </c>
     </row>
     <row r="294">
-      <c r="A294" s="1" t="n">
+      <c r="A294" t="n">
         <v>292</v>
       </c>
       <c r="B294" t="inlineStr">
@@ -8666,11 +8654,11 @@
         <v>1528.27</v>
       </c>
       <c r="H294" t="n">
-        <v>-0.0398266770978049</v>
+        <v>-0.03982667709780496</v>
       </c>
     </row>
     <row r="295">
-      <c r="A295" s="1" t="n">
+      <c r="A295" t="n">
         <v>293</v>
       </c>
       <c r="B295" t="inlineStr">
@@ -8694,11 +8682,11 @@
         <v>1496.183333333334</v>
       </c>
       <c r="H295" t="n">
-        <v>-0.1295356345571325</v>
+        <v>-0.1295356345571326</v>
       </c>
     </row>
     <row r="296">
-      <c r="A296" s="1" t="n">
+      <c r="A296" t="n">
         <v>294</v>
       </c>
       <c r="B296" t="inlineStr">
@@ -8726,7 +8714,7 @@
       </c>
     </row>
     <row r="297">
-      <c r="A297" s="1" t="n">
+      <c r="A297" t="n">
         <v>295</v>
       </c>
       <c r="B297" t="inlineStr">
@@ -8750,11 +8738,11 @@
         <v>1750.940000000001</v>
       </c>
       <c r="H297" t="n">
-        <v>-0.0651567937825845</v>
+        <v>-0.06515679378258454</v>
       </c>
     </row>
     <row r="298">
-      <c r="A298" s="1" t="n">
+      <c r="A298" t="n">
         <v>296</v>
       </c>
       <c r="B298" t="inlineStr">
@@ -8782,7 +8770,7 @@
       </c>
     </row>
     <row r="299">
-      <c r="A299" s="1" t="n">
+      <c r="A299" t="n">
         <v>297</v>
       </c>
       <c r="B299" t="inlineStr">
@@ -8810,7 +8798,7 @@
       </c>
     </row>
     <row r="300">
-      <c r="A300" s="1" t="n">
+      <c r="A300" t="n">
         <v>298</v>
       </c>
       <c r="B300" t="inlineStr">
@@ -8838,7 +8826,7 @@
       </c>
     </row>
     <row r="301">
-      <c r="A301" s="1" t="n">
+      <c r="A301" t="n">
         <v>299</v>
       </c>
       <c r="B301" t="inlineStr">
@@ -8862,11 +8850,11 @@
         <v>1554.923333333334</v>
       </c>
       <c r="H301" t="n">
-        <v>-0.0256723211610371</v>
+        <v>-0.02567232116103713</v>
       </c>
     </row>
     <row r="302">
-      <c r="A302" s="1" t="n">
+      <c r="A302" t="n">
         <v>300</v>
       </c>
       <c r="B302" t="inlineStr">
@@ -8890,11 +8878,11 @@
         <v>1307.120000000001</v>
       </c>
       <c r="H302" t="n">
-        <v>0.0835119179993126</v>
+        <v>0.08351191799931268</v>
       </c>
     </row>
     <row r="303">
-      <c r="A303" s="1" t="n">
+      <c r="A303" t="n">
         <v>301</v>
       </c>
       <c r="B303" t="inlineStr">
@@ -8918,11 +8906,11 @@
         <v>1181.096666666667</v>
       </c>
       <c r="H303" t="n">
-        <v>-0.0141071989235255</v>
+        <v>-0.01410719892352552</v>
       </c>
     </row>
     <row r="304">
-      <c r="A304" s="1" t="n">
+      <c r="A304" t="n">
         <v>302</v>
       </c>
       <c r="B304" t="inlineStr">
@@ -8950,7 +8938,7 @@
       </c>
     </row>
     <row r="305">
-      <c r="A305" s="1" t="n">
+      <c r="A305" t="n">
         <v>303</v>
       </c>
       <c r="B305" t="inlineStr">
@@ -8974,11 +8962,11 @@
         <v>1147.696666666667</v>
       </c>
       <c r="H305" t="n">
-        <v>-0.0677954326141977</v>
+        <v>-0.06779543261419774</v>
       </c>
     </row>
     <row r="306">
-      <c r="A306" s="1" t="n">
+      <c r="A306" t="n">
         <v>304</v>
       </c>
       <c r="B306" t="inlineStr">
@@ -9002,11 +8990,11 @@
         <v>1188.170000000001</v>
       </c>
       <c r="H306" t="n">
-        <v>0.1272022580141991</v>
+        <v>0.1272022580141992</v>
       </c>
     </row>
     <row r="307">
-      <c r="A307" s="1" t="n">
+      <c r="A307" t="n">
         <v>305</v>
       </c>
       <c r="B307" t="inlineStr">
@@ -9034,7 +9022,7 @@
       </c>
     </row>
     <row r="308">
-      <c r="A308" s="1" t="n">
+      <c r="A308" t="n">
         <v>306</v>
       </c>
       <c r="B308" t="inlineStr">
@@ -9058,11 +9046,11 @@
         <v>1284.690000000001</v>
       </c>
       <c r="H308" t="n">
-        <v>0.0513094697556761</v>
+        <v>0.05130946975567618</v>
       </c>
     </row>
     <row r="309">
-      <c r="A309" s="1" t="n">
+      <c r="A309" t="n">
         <v>307</v>
       </c>
       <c r="B309" t="inlineStr">
@@ -9080,17 +9068,17 @@
         <v>15466</v>
       </c>
       <c r="F309" t="n">
-        <v>2407.709677419354</v>
+        <v>2407.709677419355</v>
       </c>
       <c r="G309" t="n">
         <v>1361.676666666667</v>
       </c>
       <c r="H309" t="n">
-        <v>0.2981882012691554</v>
+        <v>0.2981882012691555</v>
       </c>
     </row>
     <row r="310">
-      <c r="A310" s="1" t="n">
+      <c r="A310" t="n">
         <v>308</v>
       </c>
       <c r="B310" t="inlineStr">
@@ -9114,11 +9102,11 @@
         <v>1459.266666666667</v>
       </c>
       <c r="H310" t="n">
-        <v>-0.2158579951215211</v>
+        <v>-0.2158579951215212</v>
       </c>
     </row>
     <row r="311">
-      <c r="A311" s="1" t="n">
+      <c r="A311" t="n">
         <v>309</v>
       </c>
       <c r="B311" t="inlineStr">
@@ -9136,7 +9124,7 @@
         <v>15483</v>
       </c>
       <c r="F311" t="n">
-        <v>2264.290322580646</v>
+        <v>2264.290322580645</v>
       </c>
       <c r="G311" t="n">
         <v>1621.943333333334</v>
@@ -9146,7 +9134,7 @@
       </c>
     </row>
     <row r="312">
-      <c r="A312" s="1" t="n">
+      <c r="A312" t="n">
         <v>310</v>
       </c>
       <c r="B312" t="inlineStr">
@@ -9170,11 +9158,11 @@
         <v>1702.813333333334</v>
       </c>
       <c r="H312" t="n">
-        <v>0.0436036408145994</v>
+        <v>0.04360364081459944</v>
       </c>
     </row>
     <row r="313">
-      <c r="A313" s="1" t="n">
+      <c r="A313" t="n">
         <v>311</v>
       </c>
       <c r="B313" t="inlineStr">
@@ -9198,11 +9186,11 @@
         <v>1657.233333333334</v>
       </c>
       <c r="H313" t="n">
-        <v>-0.0145263739631775</v>
+        <v>-0.01452637396317757</v>
       </c>
     </row>
     <row r="314">
-      <c r="A314" s="1" t="n">
+      <c r="A314" t="n">
         <v>312</v>
       </c>
       <c r="B314" t="inlineStr">
@@ -9220,17 +9208,17 @@
         <v>15584</v>
       </c>
       <c r="F314" t="n">
-        <v>2151.290322580646</v>
+        <v>2151.290322580645</v>
       </c>
       <c r="G314" t="n">
         <v>1628.130000000001</v>
       </c>
       <c r="H314" t="n">
-        <v>-0.0826675915319724</v>
+        <v>-0.08266759153197245</v>
       </c>
     </row>
     <row r="315">
-      <c r="A315" s="1" t="n">
+      <c r="A315" t="n">
         <v>313</v>
       </c>
       <c r="B315" t="inlineStr">
@@ -9254,11 +9242,11 @@
         <v>1542.590000000001</v>
       </c>
       <c r="H315" t="n">
-        <v>0.0934219856676872</v>
+        <v>0.09342198566768722</v>
       </c>
     </row>
     <row r="316">
-      <c r="A316" s="1" t="n">
+      <c r="A316" t="n">
         <v>314</v>
       </c>
       <c r="B316" t="inlineStr">
@@ -9282,11 +9270,11 @@
         <v>1795.396666666667</v>
       </c>
       <c r="H316" t="n">
-        <v>0.0900345928888495</v>
+        <v>0.09003459288884952</v>
       </c>
     </row>
     <row r="317">
-      <c r="A317" s="1" t="n">
+      <c r="A317" t="n">
         <v>315</v>
       </c>
       <c r="B317" t="inlineStr">
@@ -9310,11 +9298,11 @@
         <v>1636.940000000001</v>
       </c>
       <c r="H317" t="n">
-        <v>-0.1383778032869501</v>
+        <v>-0.1383778032869502</v>
       </c>
     </row>
     <row r="318">
-      <c r="A318" s="1" t="n">
+      <c r="A318" t="n">
         <v>316</v>
       </c>
       <c r="B318" t="inlineStr">
@@ -9338,11 +9326,11 @@
         <v>1533.873333333334</v>
       </c>
       <c r="H318" t="n">
-        <v>0.0584258556418026</v>
+        <v>0.05842585564180269</v>
       </c>
     </row>
     <row r="319">
-      <c r="A319" s="1" t="n">
+      <c r="A319" t="n">
         <v>317</v>
       </c>
       <c r="B319" t="inlineStr">
@@ -9370,7 +9358,7 @@
       </c>
     </row>
     <row r="320">
-      <c r="A320" s="1" t="n">
+      <c r="A320" t="n">
         <v>318</v>
       </c>
       <c r="B320" t="inlineStr">
@@ -9394,11 +9382,11 @@
         <v>1541.863333333334</v>
       </c>
       <c r="H320" t="n">
-        <v>0.3229700088670912</v>
+        <v>0.3229700088670913</v>
       </c>
     </row>
     <row r="321">
-      <c r="A321" s="1" t="n">
+      <c r="A321" t="n">
         <v>319</v>
       </c>
       <c r="B321" t="inlineStr">
@@ -9422,11 +9410,11 @@
         <v>1865.63</v>
       </c>
       <c r="H321" t="n">
-        <v>-0.0036731788036995</v>
+        <v>-0.003673178803699551</v>
       </c>
     </row>
     <row r="322">
-      <c r="A322" s="1" t="n">
+      <c r="A322" t="n">
         <v>320</v>
       </c>
       <c r="B322" t="inlineStr">
@@ -9450,11 +9438,11 @@
         <v>1692.773333333334</v>
       </c>
       <c r="H322" t="n">
-        <v>-0.1012979162656678</v>
+        <v>-0.1012979162656679</v>
       </c>
     </row>
     <row r="323">
-      <c r="A323" s="1" t="n">
+      <c r="A323" t="n">
         <v>321</v>
       </c>
       <c r="B323" t="inlineStr">
@@ -9475,14 +9463,14 @@
         <v>2775.903225806452</v>
       </c>
       <c r="G323" t="n">
-        <v>1876.573333333333</v>
+        <v>1876.573333333334</v>
       </c>
       <c r="H323" t="n">
-        <v>0.0616802125703455</v>
+        <v>0.06168021257034551</v>
       </c>
     </row>
     <row r="324">
-      <c r="A324" s="1" t="n">
+      <c r="A324" t="n">
         <v>322</v>
       </c>
       <c r="B324" t="inlineStr">
@@ -9510,7 +9498,7 @@
       </c>
     </row>
     <row r="325">
-      <c r="A325" s="1" t="n">
+      <c r="A325" t="n">
         <v>323</v>
       </c>
       <c r="B325" t="inlineStr">
@@ -9534,11 +9522,11 @@
         <v>1970.653333333334</v>
       </c>
       <c r="H325" t="n">
-        <v>0.0411939837561976</v>
+        <v>0.04119398375619765</v>
       </c>
     </row>
     <row r="326">
-      <c r="A326" s="1" t="n">
+      <c r="A326" t="n">
         <v>324</v>
       </c>
       <c r="B326" t="inlineStr">
@@ -9562,11 +9550,11 @@
         <v>1690.163333333334</v>
       </c>
       <c r="H326" t="n">
-        <v>0.0552203354229461</v>
+        <v>0.05522033542294613</v>
       </c>
     </row>
     <row r="327">
-      <c r="A327" s="1" t="n">
+      <c r="A327" t="n">
         <v>325</v>
       </c>
       <c r="B327" t="inlineStr">
@@ -9594,7 +9582,7 @@
       </c>
     </row>
     <row r="328">
-      <c r="A328" s="1" t="n">
+      <c r="A328" t="n">
         <v>326</v>
       </c>
       <c r="B328" t="inlineStr">
@@ -9622,7 +9610,7 @@
       </c>
     </row>
     <row r="329">
-      <c r="A329" s="1" t="n">
+      <c r="A329" t="n">
         <v>327</v>
       </c>
       <c r="B329" t="inlineStr">
@@ -9646,14 +9634,14 @@
         <v>1645.700000000001</v>
       </c>
       <c r="H329" t="n">
-        <v>-0.1557905876472954</v>
+        <v>-0.1557905876472955</v>
       </c>
     </row>
     <row r="330">
-      <c r="A330" s="1" t="n">
+      <c r="A330" t="n">
         <v>328</v>
       </c>
-      <c r="B330" s="2" t="inlineStr">
+      <c r="B330" s="1" t="inlineStr">
         <is>
           <t>2047-05</t>
         </is>
@@ -9674,7 +9662,7 @@
         <v>1362.466666666667</v>
       </c>
       <c r="H330" t="n">
-        <v>-0.4179233980225065</v>
+        <v>-0.4179233980225066</v>
       </c>
     </row>
   </sheetData>

</xml_diff>